<commit_message>
Update data and fix AHP horário scoring for nighttime competitions
- Fetch updated dPartidas.xlsx and fIngressos.xlsx from colleague's branch
- AHP: Libertadores, Copa do Brasil and Sulamericana use a nighttime horário
  table where 21:30 = 5 (prime time), replacing the default daytime table
  where 21:30 = 2

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P83"/>
+  <dimension ref="A1:P81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -568,7 +568,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30/10/2024</t>
+          <t>18/09/2024</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -581,12 +581,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Peñarol</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SEMIS</t>
+          <t>QUARTAS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -603,10 +603,10 @@
         <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
         <v>4</v>
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>4.2823</v>
+        <v>4.2257</v>
       </c>
     </row>
     <row r="4">
@@ -632,39 +632,39 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>07/12/2025</t>
+          <t>23/10/2024</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Peñarol</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>SEMIS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" t="n">
         <v>5</v>
@@ -673,10 +673,10 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N4" t="n">
         <v>3</v>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>4.132</v>
+        <v>4.2232</v>
       </c>
     </row>
     <row r="5">
@@ -696,7 +696,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>17/08/2025</t>
+          <t>07/12/2025</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -709,12 +709,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -724,34 +724,34 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I5" t="n">
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L5" t="n">
         <v>5</v>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4.0179</v>
+        <v>4.132</v>
       </c>
     </row>
     <row r="6">
@@ -760,7 +760,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03/04/2024</t>
+          <t>06/03/2024</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -773,12 +773,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Junior de Barranquilla</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -798,13 +798,13 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L6" t="n">
         <v>4</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N6" t="n">
         <v>5</v>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>4.0085</v>
+        <v>4.1276</v>
       </c>
     </row>
     <row r="7">
@@ -824,62 +824,62 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>18/09/2024</t>
+          <t>17/08/2025</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M7" t="n">
         <v>4</v>
       </c>
       <c r="N7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>3.9716</v>
+        <v>4.0179</v>
       </c>
     </row>
     <row r="8">
@@ -888,7 +888,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>25/09/2024</t>
+          <t>03/04/2024</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -901,12 +901,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Junior de Barranquilla</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -916,34 +916,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I8" t="n">
         <v>5</v>
       </c>
       <c r="J8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
         <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>3.9716</v>
+        <v>4.0085</v>
       </c>
     </row>
     <row r="9">
@@ -952,7 +952,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>23/10/2024</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -960,54 +960,54 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Peñarol</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SEMIS</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>3.9691</v>
+        <v>3.9343</v>
       </c>
     </row>
     <row r="10">
@@ -1016,11 +1016,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>03/08/2025</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1029,49 +1029,49 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I10" t="n">
         <v>4</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
         <v>4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>3.9343</v>
+        <v>3.8741</v>
       </c>
     </row>
     <row r="11">
@@ -1080,11 +1080,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>03/08/2025</t>
+          <t>19/06/2024</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Athlético</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -1118,24 +1118,24 @@
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>3.8741</v>
+        <v>3.8675</v>
       </c>
     </row>
     <row r="12">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06/03/2024</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1182,24 +1182,24 @@
         <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L12" t="n">
         <v>4</v>
       </c>
       <c r="M12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.8735</v>
+        <v>3.8647</v>
       </c>
     </row>
     <row r="13">
@@ -1208,62 +1208,62 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>19/06/2024</t>
+          <t>11/09/2025</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Athlético</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>QUARTAS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>3.8675</v>
+        <v>3.8436</v>
       </c>
     </row>
     <row r="14">
@@ -1528,11 +1528,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>14/08/2025</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1541,22 +1541,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Universitario</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1566,10 +1566,10 @@
         <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M18" t="n">
         <v>3</v>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>3.7646</v>
+        <v>3.6953</v>
       </c>
     </row>
     <row r="19">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>05/05/2024</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1600,54 +1600,54 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Universitario</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M19" t="n">
         <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>3.6953</v>
+        <v>3.6569</v>
       </c>
     </row>
     <row r="20">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05/05/2024</t>
+          <t>07/07/2024</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1684,14 +1684,14 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
         <v>3</v>
@@ -1703,15 +1703,15 @@
         <v>3</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>3.6569</v>
+        <v>3.6544</v>
       </c>
     </row>
     <row r="21">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07/07/2024</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1728,31 +1728,31 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J21" t="n">
         <v>3</v>
@@ -1761,21 +1761,21 @@
         <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M21" t="n">
         <v>3</v>
       </c>
       <c r="N21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>3.6544</v>
+        <v>3.6264</v>
       </c>
     </row>
     <row r="22">
@@ -1784,62 +1784,62 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>14/05/2025</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Estudiantes</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>3.6264</v>
+        <v>3.6043</v>
       </c>
     </row>
     <row r="23">
@@ -1848,25 +1848,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08/05/2024</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1876,34 +1876,34 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L23" t="n">
         <v>4</v>
       </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>3.6106</v>
+        <v>3.6021</v>
       </c>
     </row>
     <row r="24">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>05/11/2025</t>
+          <t>14/08/2025</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1920,54 +1920,54 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
         <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>3.6021</v>
+        <v>3.5952</v>
       </c>
     </row>
     <row r="25">
@@ -1976,62 +1976,62 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11/09/2025</t>
+          <t>17/03/2024</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>3.5895</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="26">
@@ -2040,62 +2040,62 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>17/03/2024</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K26" t="n">
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>3.58</v>
+        <v>3.5543</v>
       </c>
     </row>
     <row r="27">
@@ -2104,11 +2104,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2117,38 +2117,38 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I27" t="n">
         <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N27" t="n">
         <v>4</v>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>3.5543</v>
+        <v>3.5303</v>
       </c>
     </row>
     <row r="28">
@@ -2168,11 +2168,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2181,35 +2181,35 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I28" t="n">
         <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M28" t="n">
         <v>4</v>
@@ -2219,11 +2219,11 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.5303</v>
+        <v>3.5045</v>
       </c>
     </row>
     <row r="29">
@@ -2232,62 +2232,62 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>28/02/2024</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29" t="n">
         <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.5045</v>
+        <v>3.5012</v>
       </c>
     </row>
     <row r="30">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>14/05/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2496,43 +2496,43 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Estudiantes</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J33" t="n">
         <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N33" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.3502</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="34">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2560,43 +2560,43 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.3437</v>
+        <v>3.3127</v>
       </c>
     </row>
     <row r="35">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2624,17 +2624,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2644,14 +2644,14 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K35" t="n">
         <v>3</v>
@@ -2660,7 +2660,7 @@
         <v>4</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N35" t="n">
         <v>4</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.3127</v>
+        <v>3.2939</v>
       </c>
     </row>
     <row r="36">
@@ -2680,51 +2680,51 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.2939</v>
+        <v>3.2629</v>
       </c>
     </row>
     <row r="37">
@@ -2744,62 +2744,62 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>18/10/2024</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Criciúma</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sexta-feira</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K37" t="n">
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.2629</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="38">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2821,22 +2821,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I38" t="n">
@@ -2872,25 +2872,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2900,17 +2900,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2515</v>
+        <v>3.2512</v>
       </c>
     </row>
     <row r="40">
@@ -2936,62 +2936,62 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Aurora</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2471</v>
+        <v>3.2452</v>
       </c>
     </row>
     <row r="41">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>27/02/2025</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -3008,40 +3008,40 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Recopa</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Racing</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>FINAL</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K41" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M41" t="n">
         <v>4</v>
@@ -3051,11 +3051,11 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P41" t="n">
-        <v>3.2452</v>
+        <v>3.2426</v>
       </c>
     </row>
     <row r="42">
@@ -3064,45 +3064,45 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27/02/2025</t>
+          <t>14/09/2024</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Recopa</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Racing</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>FINAL</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L42" t="n">
         <v>3</v>
@@ -3111,15 +3111,15 @@
         <v>4</v>
       </c>
       <c r="N42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2426</v>
+        <v>3.1913</v>
       </c>
     </row>
     <row r="43">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>14/09/2024</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -3141,22 +3141,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -3169,21 +3169,21 @@
         <v>3</v>
       </c>
       <c r="L43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N43" t="n">
         <v>3</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.1913</v>
+        <v>3.1908</v>
       </c>
     </row>
     <row r="44">
@@ -3192,11 +3192,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>17/09/2025</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>17/09/2025</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -3269,12 +3269,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -3294,13 +3294,13 @@
         <v>3</v>
       </c>
       <c r="K45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
       </c>
       <c r="M45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N45" t="n">
         <v>3</v>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>3.1908</v>
+        <v>3.1564</v>
       </c>
     </row>
     <row r="46">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>31/08/2024</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3333,22 +3333,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -3358,10 +3358,10 @@
         <v>3</v>
       </c>
       <c r="K46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M46" t="n">
         <v>3</v>
@@ -3371,11 +3371,11 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.1564</v>
+        <v>3.141</v>
       </c>
     </row>
     <row r="47">
@@ -3384,11 +3384,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>31/08/2024</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3397,49 +3397,49 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I47" t="n">
         <v>4</v>
       </c>
       <c r="J47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L47" t="n">
         <v>3</v>
       </c>
       <c r="M47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>3.141</v>
+        <v>3.1091</v>
       </c>
     </row>
     <row r="48">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3461,49 +3461,49 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I48" t="n">
         <v>4</v>
       </c>
       <c r="J48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>3.1091</v>
+        <v>3.0907</v>
       </c>
     </row>
     <row r="49">
@@ -3512,11 +3512,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3525,49 +3525,49 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I49" t="n">
         <v>4</v>
       </c>
       <c r="J49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="n">
         <v>3</v>
       </c>
       <c r="L49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>3.0907</v>
+        <v>2.9936</v>
       </c>
     </row>
     <row r="50">
@@ -3576,11 +3576,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3589,12 +3589,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3611,27 +3611,27 @@
         <v>5</v>
       </c>
       <c r="J50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K50" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
       </c>
       <c r="M50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N50" t="n">
         <v>3</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2.9971</v>
+        <v>2.9908</v>
       </c>
     </row>
     <row r="51">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -3648,54 +3648,54 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L51" t="n">
+        <v>4</v>
+      </c>
+      <c r="M51" t="n">
+        <v>4</v>
+      </c>
+      <c r="N51" t="n">
         <v>1</v>
       </c>
-      <c r="M51" t="n">
-        <v>4</v>
-      </c>
-      <c r="N51" t="n">
-        <v>4</v>
-      </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>2.9936</v>
+        <v>2.9754</v>
       </c>
     </row>
     <row r="52">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3712,43 +3712,43 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="n">
         <v>5</v>
       </c>
       <c r="L52" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N52" t="n">
         <v>3</v>
@@ -3759,7 +3759,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2.9682</v>
+        <v>2.9692</v>
       </c>
     </row>
     <row r="53">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>31/03/2024</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3781,12 +3781,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -3806,24 +3806,24 @@
         <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L53" t="n">
         <v>5</v>
       </c>
       <c r="M53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P53" t="n">
-        <v>2.9611</v>
+        <v>2.9682</v>
       </c>
     </row>
     <row r="54">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>27/01/2024</t>
+          <t>31/03/2024</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3845,22 +3845,22 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -3870,10 +3870,10 @@
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L54" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M54" t="n">
         <v>1</v>
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2.9303</v>
+        <v>2.9611</v>
       </c>
     </row>
     <row r="55">
@@ -3896,11 +3896,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>11/01/2025</t>
+          <t>27/01/2024</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3909,12 +3909,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Maricá</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3960,25 +3960,25 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>11/01/2025</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Maricá</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3988,34 +3988,34 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J56" t="n">
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L56" t="n">
         <v>3</v>
       </c>
       <c r="M56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2.8806</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="57">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4032,31 +4032,31 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J57" t="n">
         <v>2</v>
@@ -4065,21 +4065,21 @@
         <v>3</v>
       </c>
       <c r="L57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.861</v>
+        <v>2.8806</v>
       </c>
     </row>
     <row r="58">
@@ -4088,51 +4088,51 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>18/08/2024</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Nacional de Potosí</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J58" t="n">
         <v>3</v>
       </c>
       <c r="K58" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N58" t="n">
         <v>1</v>
@@ -4143,7 +4143,7 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2.7651</v>
+        <v>2.8748</v>
       </c>
     </row>
     <row r="59">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>24/01/2026</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -4165,22 +4165,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -4193,7 +4193,7 @@
         <v>3</v>
       </c>
       <c r="L59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M59" t="n">
         <v>1</v>
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2.7609</v>
+        <v>2.861</v>
       </c>
     </row>
     <row r="60">
@@ -4216,62 +4216,62 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>SEMIS - TR</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K60" t="n">
         <v>3</v>
       </c>
       <c r="L60" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M60" t="n">
+        <v>4</v>
+      </c>
+      <c r="N60" t="n">
         <v>1</v>
       </c>
-      <c r="N60" t="n">
-        <v>4</v>
-      </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2.7609</v>
+        <v>2.7651</v>
       </c>
     </row>
     <row r="61">
@@ -4280,62 +4280,62 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>29/07/2025</t>
+          <t>24/01/2026</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K61" t="n">
         <v>3</v>
       </c>
       <c r="L61" t="n">
+        <v>3</v>
+      </c>
+      <c r="M61" t="n">
         <v>1</v>
       </c>
-      <c r="M61" t="n">
-        <v>2</v>
-      </c>
       <c r="N61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2.7495</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="62">
@@ -4344,62 +4344,62 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>SEMIS - TR</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J62" t="n">
         <v>2</v>
       </c>
       <c r="K62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L62" t="n">
+        <v>3</v>
+      </c>
+      <c r="M62" t="n">
         <v>1</v>
       </c>
-      <c r="M62" t="n">
-        <v>4</v>
-      </c>
       <c r="N62" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P62" t="n">
-        <v>2.7367</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="63">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>29/07/2025</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -4416,17 +4416,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -4440,10 +4440,10 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" t="n">
         <v>3</v>
@@ -4459,11 +4459,11 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P63" t="n">
-        <v>2.7208</v>
+        <v>2.7495</v>
       </c>
     </row>
     <row r="64">
@@ -4472,25 +4472,25 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -4500,23 +4500,23 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L64" t="n">
         <v>1</v>
       </c>
       <c r="M64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N64" t="n">
         <v>3</v>
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>2.7151</v>
+        <v>2.7208</v>
       </c>
     </row>
     <row r="65">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>15/02/2026</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -4608,54 +4608,54 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Nacional de Potosí</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>Quartas</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M66" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>D+D+D</t>
         </is>
       </c>
       <c r="P66" t="n">
-        <v>2.6207</v>
+        <v>2.5653</v>
       </c>
     </row>
     <row r="67">
@@ -4664,62 +4664,62 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>15/02/2026</t>
+          <t>16/07/2025</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Quartas</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>D+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>2.5653</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="68">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>16/07/2025</t>
+          <t>20/09/2025</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -4741,22 +4741,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -4766,10 +4766,10 @@
         <v>3</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M68" t="n">
         <v>3</v>
@@ -4779,11 +4779,11 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+E+D</t>
         </is>
       </c>
       <c r="P68" t="n">
-        <v>2.53</v>
+        <v>2.5146</v>
       </c>
     </row>
     <row r="69">
@@ -4792,62 +4792,62 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>20/09/2025</t>
+          <t>30/01/2024</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Portuguesa</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>E+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P69" t="n">
-        <v>2.5146</v>
+        <v>2.476</v>
       </c>
     </row>
     <row r="70">
@@ -4856,11 +4856,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>30/01/2024</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -4869,22 +4869,22 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Portuguesa</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>FINAL - TR</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I70" t="n">
@@ -4894,24 +4894,24 @@
         <v>2</v>
       </c>
       <c r="K70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M70" t="n">
         <v>1</v>
       </c>
       <c r="N70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P70" t="n">
-        <v>2.476</v>
+        <v>2.4477</v>
       </c>
     </row>
     <row r="71">
@@ -4920,39 +4920,39 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>21/04/2024</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>FINAL - TR</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I71" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J71" t="n">
         <v>2</v>
@@ -4961,21 +4961,21 @@
         <v>3</v>
       </c>
       <c r="L71" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M71" t="n">
+        <v>2</v>
+      </c>
+      <c r="N71" t="n">
         <v>1</v>
       </c>
-      <c r="N71" t="n">
-        <v>3</v>
-      </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P71" t="n">
-        <v>2.4477</v>
+        <v>2.3538</v>
       </c>
     </row>
     <row r="72">
@@ -4984,11 +4984,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>21/04/2024</t>
+          <t>26/04/2025</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4997,22 +4997,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -5025,21 +5025,21 @@
         <v>3</v>
       </c>
       <c r="L72" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M72" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N72" t="n">
         <v>1</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P72" t="n">
-        <v>2.3538</v>
+        <v>2.2542</v>
       </c>
     </row>
     <row r="73">
@@ -5048,11 +5048,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -5061,22 +5061,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -5089,21 +5089,21 @@
         <v>3</v>
       </c>
       <c r="L73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M73" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N73" t="n">
         <v>1</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>2.2542</v>
+        <v>2.2537</v>
       </c>
     </row>
     <row r="74">
@@ -5112,11 +5112,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>05/04/2025</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -5125,22 +5125,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I74" t="n">
@@ -5153,7 +5153,7 @@
         <v>3</v>
       </c>
       <c r="L74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M74" t="n">
         <v>2</v>
@@ -5163,11 +5163,11 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P74" t="n">
-        <v>2.2537</v>
+        <v>2.1536</v>
       </c>
     </row>
     <row r="75">
@@ -5176,11 +5176,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>05/04/2025</t>
+          <t>18/04/2024</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Atlético-GO</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5199,12 +5199,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -5214,7 +5214,7 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L75" t="n">
         <v>3</v>
@@ -5227,11 +5227,11 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P75" t="n">
-        <v>2.1536</v>
+        <v>2.0689</v>
       </c>
     </row>
     <row r="76">
@@ -5240,51 +5240,51 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>18/04/2024</t>
+          <t>26/01/2025</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Atlético-GO</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I76" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J76" t="n">
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L76" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N76" t="n">
         <v>1</v>
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>2.0689</v>
+        <v>2.0215</v>
       </c>
     </row>
     <row r="77">
@@ -5304,7 +5304,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>26/01/2025</t>
+          <t>29/01/2025</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -5317,22 +5317,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -5342,13 +5342,13 @@
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M77" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N77" t="n">
         <v>1</v>
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>2.0215</v>
+        <v>1.9876</v>
       </c>
     </row>
     <row r="78">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>29/01/2025</t>
+          <t>22/01/2025</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -5381,12 +5381,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -5412,7 +5412,7 @@
         <v>4</v>
       </c>
       <c r="M78" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N78" t="n">
         <v>1</v>
@@ -5423,7 +5423,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>1.9876</v>
+        <v>1.8367</v>
       </c>
     </row>
     <row r="79">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>22/01/2025</t>
+          <t>14/01/2025</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -5445,22 +5445,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Portuguesa</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I79" t="n">
@@ -5470,10 +5470,10 @@
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M79" t="n">
         <v>1</v>
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>1.8367</v>
+        <v>1.6211</v>
       </c>
     </row>
     <row r="80">
@@ -5496,11 +5496,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>14/01/2025</t>
+          <t>17/01/2024</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -5509,22 +5509,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Portuguesa</t>
+          <t>Madureira</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I80" t="n">
@@ -5537,22 +5537,14 @@
         <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M80" t="n">
         <v>1</v>
       </c>
-      <c r="N80" t="n">
-        <v>1</v>
-      </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>V+D+D</t>
-        </is>
-      </c>
-      <c r="P80" t="n">
-        <v>1.6211</v>
-      </c>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -5560,7 +5552,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>17/01/2024</t>
+          <t>20/01/2024</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -5573,22 +5565,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Madureira</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I81" t="n">
@@ -5598,10 +5590,10 @@
         <v>2</v>
       </c>
       <c r="K81" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M81" t="n">
         <v>1</v>
@@ -5609,118 +5601,6 @@
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>20/01/2024</t>
-        </is>
-      </c>
-      <c r="C82" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Carioca</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Bangu</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="I82" t="n">
-        <v>2</v>
-      </c>
-      <c r="J82" t="n">
-        <v>2</v>
-      </c>
-      <c r="K82" t="n">
-        <v>5</v>
-      </c>
-      <c r="L82" t="n">
-        <v>3</v>
-      </c>
-      <c r="M82" t="n">
-        <v>1</v>
-      </c>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>14/08/2024</t>
-        </is>
-      </c>
-      <c r="C83" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Palmeiras</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>OITAVAS</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Quarta-feira</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="n">
-        <v>3</v>
-      </c>
-      <c r="K83" t="n">
-        <v>2</v>
-      </c>
-      <c r="L83" t="n">
-        <v>4</v>
-      </c>
-      <c r="M83" t="n">
-        <v>4</v>
-      </c>
-      <c r="N83" t="n">
-        <v>1</v>
-      </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t>V+D+D</t>
-        </is>
-      </c>
-      <c r="P83" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
AHP: Quarta-feira = 5 para Libertadores, Copa do Brasil e Sulamericana
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -609,7 +609,7 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M3" t="n">
         <v>4</v>
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>4.2257</v>
+        <v>4.3258</v>
       </c>
     </row>
     <row r="4">
@@ -673,7 +673,7 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4" t="n">
         <v>4</v>
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>4.2232</v>
+        <v>4.3233</v>
       </c>
     </row>
     <row r="5">
@@ -696,42 +696,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>07/12/2025</t>
+          <t>06/03/2024</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
         <v>5</v>
@@ -740,18 +740,18 @@
         <v>5</v>
       </c>
       <c r="M5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4.132</v>
+        <v>4.2277</v>
       </c>
     </row>
     <row r="6">
@@ -760,62 +760,62 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06/03/2024</t>
+          <t>07/12/2025</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K6" t="n">
         <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>4.1276</v>
+        <v>4.132</v>
       </c>
     </row>
     <row r="7">
@@ -824,39 +824,39 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17/08/2025</t>
+          <t>03/04/2024</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Junior de Barranquilla</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -868,7 +868,7 @@
         <v>5</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" t="n">
         <v>5</v>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>4.0179</v>
+        <v>4.1086</v>
       </c>
     </row>
     <row r="8">
@@ -888,39 +888,39 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03/04/2024</t>
+          <t>17/08/2025</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Junior de Barranquilla</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
@@ -929,10 +929,10 @@
         <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N8" t="n">
         <v>5</v>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>4.0085</v>
+        <v>4.0179</v>
       </c>
     </row>
     <row r="9">
@@ -952,7 +952,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -960,40 +960,40 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
         <v>5</v>
       </c>
       <c r="L9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
         <v>3</v>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>3.9343</v>
+        <v>3.9648</v>
       </c>
     </row>
     <row r="10">
@@ -1016,11 +1016,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>03/08/2025</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1029,49 +1029,49 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I10" t="n">
         <v>4</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
         <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" t="n">
         <v>4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>3.8741</v>
+        <v>3.9343</v>
       </c>
     </row>
     <row r="11">
@@ -1080,11 +1080,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>19/06/2024</t>
+          <t>03/08/2025</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Athlético</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -1118,24 +1118,24 @@
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>3.8675</v>
+        <v>3.8741</v>
       </c>
     </row>
     <row r="12">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08/05/2024</t>
+          <t>19/06/2024</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Athlético</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1172,17 +1172,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
         <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L12" t="n">
         <v>4</v>
@@ -1191,15 +1191,15 @@
         <v>3</v>
       </c>
       <c r="N12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.8647</v>
+        <v>3.8675</v>
       </c>
     </row>
     <row r="13">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>20/07/2024</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1408,31 +1408,31 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Universitario</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
@@ -1441,21 +1441,21 @@
         <v>3</v>
       </c>
       <c r="L16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M16" t="n">
         <v>3</v>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>3.7674</v>
+        <v>3.7954</v>
       </c>
     </row>
     <row r="17">
@@ -1464,11 +1464,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>22/11/2025</t>
+          <t>20/07/2024</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1477,12 +1477,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Grêmio</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1492,14 +1492,14 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I17" t="n">
         <v>4</v>
       </c>
       <c r="J17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
         <v>3</v>
@@ -1511,15 +1511,15 @@
         <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>3.7649</v>
+        <v>3.7674</v>
       </c>
     </row>
     <row r="18">
@@ -1528,48 +1528,48 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>22/11/2025</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Universitario</t>
+          <t>Grêmio</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K18" t="n">
         <v>3</v>
       </c>
       <c r="L18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
         <v>3</v>
@@ -1579,11 +1579,11 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>3.6953</v>
+        <v>3.7649</v>
       </c>
     </row>
     <row r="19">
@@ -1592,20 +1592,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>05/05/2024</t>
+          <t>14/05/2025</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Estudiantes</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1615,39 +1615,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J19" t="n">
         <v>2</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L19" t="n">
         <v>5</v>
       </c>
       <c r="M19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>3.6569</v>
+        <v>3.7044</v>
       </c>
     </row>
     <row r="20">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07/07/2024</t>
+          <t>05/05/2024</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1684,14 +1684,14 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="n">
         <v>3</v>
@@ -1703,15 +1703,15 @@
         <v>3</v>
       </c>
       <c r="N20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>3.6544</v>
+        <v>3.6569</v>
       </c>
     </row>
     <row r="21">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>07/07/2024</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1728,31 +1728,31 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J21" t="n">
         <v>3</v>
@@ -1761,21 +1761,21 @@
         <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M21" t="n">
         <v>3</v>
       </c>
       <c r="N21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>3.6264</v>
+        <v>3.6544</v>
       </c>
     </row>
     <row r="22">
@@ -1784,62 +1784,62 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>14/05/2025</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Estudiantes</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>3.6043</v>
+        <v>3.6264</v>
       </c>
     </row>
     <row r="23">
@@ -1912,11 +1912,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>14/08/2025</t>
+          <t>28/02/2024</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1925,22 +1925,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -1950,24 +1950,24 @@
         <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>3.5952</v>
+        <v>3.6013</v>
       </c>
     </row>
     <row r="25">
@@ -1976,62 +1976,62 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>17/03/2024</t>
+          <t>14/08/2025</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K25" t="n">
         <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>3.58</v>
+        <v>3.5952</v>
       </c>
     </row>
     <row r="26">
@@ -2040,62 +2040,62 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>17/03/2024</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K26" t="n">
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>3.5543</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="27">
@@ -2104,11 +2104,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2117,38 +2117,38 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I27" t="n">
         <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N27" t="n">
         <v>4</v>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>3.5303</v>
+        <v>3.5543</v>
       </c>
     </row>
     <row r="28">
@@ -2168,11 +2168,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2181,35 +2181,35 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I28" t="n">
         <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M28" t="n">
         <v>4</v>
@@ -2219,11 +2219,11 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.5045</v>
+        <v>3.5303</v>
       </c>
     </row>
     <row r="29">
@@ -2232,62 +2232,62 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aurora</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J29" t="n">
         <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.5012</v>
+        <v>3.5045</v>
       </c>
     </row>
     <row r="30">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2496,34 +2496,34 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" t="n">
         <v>3</v>
@@ -2532,7 +2532,7 @@
         <v>5</v>
       </c>
       <c r="M33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N33" t="n">
         <v>4</v>
@@ -2543,7 +2543,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.3437</v>
+        <v>3.4128</v>
       </c>
     </row>
     <row r="34">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2560,43 +2560,43 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.3127</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="35">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -3520,54 +3520,54 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L49" t="n">
+        <v>5</v>
+      </c>
+      <c r="M49" t="n">
+        <v>4</v>
+      </c>
+      <c r="N49" t="n">
         <v>1</v>
       </c>
-      <c r="M49" t="n">
-        <v>4</v>
-      </c>
-      <c r="N49" t="n">
-        <v>4</v>
-      </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>2.9936</v>
+        <v>3.0755</v>
       </c>
     </row>
     <row r="50">
@@ -3576,25 +3576,25 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3604,17 +3604,17 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J50" t="n">
         <v>2</v>
       </c>
       <c r="K50" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L50" t="n">
         <v>1</v>
@@ -3623,15 +3623,15 @@
         <v>4</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2.9908</v>
+        <v>2.9936</v>
       </c>
     </row>
     <row r="51">
@@ -3640,11 +3640,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3653,17 +3653,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3675,27 +3675,27 @@
         <v>5</v>
       </c>
       <c r="J51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K51" t="n">
         <v>5</v>
       </c>
       <c r="L51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M51" t="n">
         <v>4</v>
       </c>
       <c r="N51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>2.9754</v>
+        <v>2.9908</v>
       </c>
     </row>
     <row r="52">
@@ -3704,30 +3704,30 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Nacional de Potosí</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J52" t="n">
         <v>3</v>
@@ -3745,21 +3745,21 @@
         <v>5</v>
       </c>
       <c r="L52" t="n">
+        <v>5</v>
+      </c>
+      <c r="M52" t="n">
+        <v>2</v>
+      </c>
+      <c r="N52" t="n">
         <v>1</v>
       </c>
-      <c r="M52" t="n">
-        <v>3</v>
-      </c>
-      <c r="N52" t="n">
-        <v>3</v>
-      </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2.9692</v>
+        <v>2.9749</v>
       </c>
     </row>
     <row r="53">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3776,43 +3776,43 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K53" t="n">
         <v>5</v>
       </c>
       <c r="L53" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N53" t="n">
         <v>3</v>
@@ -3823,7 +3823,7 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>2.9682</v>
+        <v>2.9692</v>
       </c>
     </row>
     <row r="54">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>31/03/2024</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3845,12 +3845,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -3870,24 +3870,24 @@
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L54" t="n">
         <v>5</v>
       </c>
       <c r="M54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2.9611</v>
+        <v>2.9682</v>
       </c>
     </row>
     <row r="55">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>27/01/2024</t>
+          <t>31/03/2024</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3909,22 +3909,22 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -3934,10 +3934,10 @@
         <v>2</v>
       </c>
       <c r="K55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L55" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M55" t="n">
         <v>1</v>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>2.9303</v>
+        <v>2.9611</v>
       </c>
     </row>
     <row r="56">
@@ -3960,11 +3960,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>11/01/2025</t>
+          <t>27/01/2024</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3973,12 +3973,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Maricá</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4024,25 +4024,25 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>11/01/2025</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Maricá</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4052,34 +4052,34 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L57" t="n">
         <v>3</v>
       </c>
       <c r="M57" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.8806</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="58">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -4096,54 +4096,54 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Nacional de Potosí</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2.8748</v>
+        <v>2.8806</v>
       </c>
     </row>
     <row r="59">

</xml_diff>

<commit_message>
AHP: Terça e Quinta = 4 para Libertadores, Copa do Brasil e Sulamericana
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -1016,39 +1016,39 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>11/09/2025</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>QUARTAS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
         <v>4</v>
@@ -1057,21 +1057,21 @@
         <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" t="n">
         <v>4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>3.9343</v>
+        <v>3.9437</v>
       </c>
     </row>
     <row r="11">
@@ -1080,11 +1080,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>03/08/2025</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1093,49 +1093,49 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I11" t="n">
         <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" t="n">
         <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N11" t="n">
         <v>4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>3.8741</v>
+        <v>3.9343</v>
       </c>
     </row>
     <row r="12">
@@ -1144,11 +1144,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>19/06/2024</t>
+          <t>03/08/2025</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1157,22 +1157,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Athlético</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -1182,24 +1182,24 @@
         <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.8675</v>
+        <v>3.8741</v>
       </c>
     </row>
     <row r="13">
@@ -1208,62 +1208,62 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11/09/2025</t>
+          <t>19/06/2024</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Athlético</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>3.8436</v>
+        <v>3.8675</v>
       </c>
     </row>
     <row r="14">
@@ -1592,62 +1592,62 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>14/05/2025</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Estudiantes</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>3.7044</v>
+        <v>3.7265</v>
       </c>
     </row>
     <row r="20">
@@ -1656,20 +1656,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05/05/2024</t>
+          <t>14/05/2025</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Estudiantes</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1679,39 +1679,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J20" t="n">
         <v>2</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L20" t="n">
         <v>5</v>
       </c>
       <c r="M20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>3.6569</v>
+        <v>3.7044</v>
       </c>
     </row>
     <row r="21">
@@ -1720,39 +1720,39 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07/07/2024</t>
+          <t>14/08/2025</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J21" t="n">
         <v>3</v>
@@ -1761,7 +1761,7 @@
         <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M21" t="n">
         <v>3</v>
@@ -1771,11 +1771,11 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>3.6544</v>
+        <v>3.6953</v>
       </c>
     </row>
     <row r="22">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>05/05/2024</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1792,40 +1792,40 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K22" t="n">
         <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>3.6264</v>
+        <v>3.6569</v>
       </c>
     </row>
     <row r="23">
@@ -1848,11 +1848,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>05/11/2025</t>
+          <t>07/07/2024</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1861,49 +1861,49 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I23" t="n">
         <v>4</v>
       </c>
       <c r="J23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K23" t="n">
         <v>3</v>
       </c>
       <c r="L23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>3.6021</v>
+        <v>3.6544</v>
       </c>
     </row>
     <row r="24">
@@ -1912,25 +1912,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Aurora</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1940,34 +1940,34 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N24" t="n">
         <v>3</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>3.6013</v>
+        <v>3.6021</v>
       </c>
     </row>
     <row r="25">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>14/08/2025</t>
+          <t>28/02/2024</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1989,22 +1989,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -2014,24 +2014,24 @@
         <v>3</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>3.5952</v>
+        <v>3.6013</v>
       </c>
     </row>
     <row r="26">
@@ -2168,25 +2168,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2200,30 +2200,30 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.5303</v>
+        <v>3.5515</v>
       </c>
     </row>
     <row r="29">
@@ -2232,11 +2232,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2245,35 +2245,35 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I29" t="n">
         <v>4</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
         <v>4</v>
@@ -2283,11 +2283,11 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.5045</v>
+        <v>3.5303</v>
       </c>
     </row>
     <row r="30">
@@ -2296,11 +2296,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>23/11/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2309,12 +2309,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2324,14 +2324,14 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I30" t="n">
         <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
         <v>3</v>
@@ -2340,18 +2340,18 @@
         <v>3</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>3.4517</v>
+        <v>3.5045</v>
       </c>
     </row>
     <row r="31">
@@ -2360,62 +2360,62 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>23/11/2024</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>3.4252</v>
+        <v>3.4517</v>
       </c>
     </row>
     <row r="32">
@@ -2424,62 +2424,62 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M32" t="n">
         <v>4</v>
       </c>
       <c r="N32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>3.4198</v>
+        <v>3.4252</v>
       </c>
     </row>
     <row r="33">
@@ -2488,62 +2488,62 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J33" t="n">
         <v>3</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N33" t="n">
         <v>4</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.4128</v>
+        <v>3.4198</v>
       </c>
     </row>
     <row r="34">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2560,34 +2560,34 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K34" t="n">
         <v>3</v>
@@ -2596,7 +2596,7 @@
         <v>5</v>
       </c>
       <c r="M34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.3437</v>
+        <v>3.4128</v>
       </c>
     </row>
     <row r="35">
@@ -2616,42 +2616,42 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K35" t="n">
         <v>3</v>
@@ -2660,7 +2660,7 @@
         <v>4</v>
       </c>
       <c r="M35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
         <v>4</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.2939</v>
+        <v>3.363</v>
       </c>
     </row>
     <row r="36">
@@ -2680,51 +2680,51 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.2629</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="37">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2757,49 +2757,49 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I37" t="n">
         <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K37" t="n">
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.2515</v>
+        <v>3.2939</v>
       </c>
     </row>
     <row r="38">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2816,17 +2816,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2836,34 +2836,34 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N38" t="n">
         <v>3</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.2515</v>
+        <v>3.2911</v>
       </c>
     </row>
     <row r="39">
@@ -2872,25 +2872,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2904,7 +2904,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J39" t="n">
         <v>3</v>
@@ -2913,7 +2913,7 @@
         <v>5</v>
       </c>
       <c r="L39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M39" t="n">
         <v>3</v>
@@ -2923,11 +2923,11 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2512</v>
+        <v>3.2695</v>
       </c>
     </row>
     <row r="40">
@@ -2936,11 +2936,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>18/10/2024</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Criciúma</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sexta-feira</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -2974,24 +2974,24 @@
         <v>4</v>
       </c>
       <c r="K40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2452</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="41">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>27/02/2025</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -3008,54 +3008,54 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Recopa</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Racing</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>FINAL</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P41" t="n">
-        <v>3.2426</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="42">
@@ -3064,11 +3064,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>14/09/2024</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -3077,49 +3077,49 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I42" t="n">
         <v>4</v>
       </c>
       <c r="J42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M42" t="n">
         <v>4</v>
       </c>
       <c r="N42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.1913</v>
+        <v>3.2452</v>
       </c>
     </row>
     <row r="43">
@@ -3128,62 +3128,62 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>27/02/2025</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Recopa</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Racing</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>FINAL</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J43" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.1908</v>
+        <v>3.2426</v>
       </c>
     </row>
     <row r="44">
@@ -3192,11 +3192,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>17/09/2025</t>
+          <t>14/09/2024</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3205,22 +3205,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -3233,21 +3233,21 @@
         <v>3</v>
       </c>
       <c r="L44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N44" t="n">
         <v>3</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>3.1908</v>
+        <v>3.1913</v>
       </c>
     </row>
     <row r="45">
@@ -3256,11 +3256,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -3294,13 +3294,13 @@
         <v>3</v>
       </c>
       <c r="K45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L45" t="n">
         <v>4</v>
       </c>
       <c r="M45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N45" t="n">
         <v>3</v>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>3.1564</v>
+        <v>3.1908</v>
       </c>
     </row>
     <row r="46">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>31/08/2024</t>
+          <t>17/09/2025</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -3333,22 +3333,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -3361,21 +3361,21 @@
         <v>3</v>
       </c>
       <c r="L46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N46" t="n">
         <v>3</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.141</v>
+        <v>3.1908</v>
       </c>
     </row>
     <row r="47">
@@ -3384,11 +3384,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3397,17 +3397,17 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3419,27 +3419,27 @@
         <v>4</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K47" t="n">
         <v>2</v>
       </c>
       <c r="L47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>3.1091</v>
+        <v>3.1564</v>
       </c>
     </row>
     <row r="48">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>31/08/2024</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3461,12 +3461,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -3492,18 +3492,18 @@
         <v>3</v>
       </c>
       <c r="M48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N48" t="n">
         <v>3</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>3.0907</v>
+        <v>3.141</v>
       </c>
     </row>
     <row r="49">
@@ -3512,30 +3512,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3544,30 +3544,30 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L49" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M49" t="n">
         <v>4</v>
       </c>
       <c r="N49" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>3.0755</v>
+        <v>3.1091</v>
       </c>
     </row>
     <row r="50">
@@ -3576,11 +3576,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -3589,49 +3589,49 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I50" t="n">
         <v>4</v>
       </c>
       <c r="J50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K50" t="n">
         <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2.9936</v>
+        <v>3.0907</v>
       </c>
     </row>
     <row r="51">
@@ -3640,11 +3640,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -3653,17 +3653,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3675,27 +3675,27 @@
         <v>5</v>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K51" t="n">
         <v>5</v>
       </c>
       <c r="L51" t="n">
+        <v>5</v>
+      </c>
+      <c r="M51" t="n">
+        <v>4</v>
+      </c>
+      <c r="N51" t="n">
         <v>1</v>
       </c>
-      <c r="M51" t="n">
-        <v>4</v>
-      </c>
-      <c r="N51" t="n">
-        <v>3</v>
-      </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>2.9908</v>
+        <v>3.0755</v>
       </c>
     </row>
     <row r="52">
@@ -3704,62 +3704,62 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>29/07/2025</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Nacional de Potosí</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J52" t="n">
         <v>3</v>
       </c>
       <c r="K52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M52" t="n">
         <v>2</v>
       </c>
       <c r="N52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2.9749</v>
+        <v>3.0498</v>
       </c>
     </row>
     <row r="53">
@@ -3768,25 +3768,25 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3796,23 +3796,23 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N53" t="n">
         <v>3</v>
@@ -3823,7 +3823,7 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>2.9692</v>
+        <v>3.0211</v>
       </c>
     </row>
     <row r="54">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3840,54 +3840,54 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J54" t="n">
         <v>2</v>
       </c>
       <c r="K54" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L54" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M54" t="n">
         <v>4</v>
       </c>
       <c r="N54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2.9682</v>
+        <v>2.9936</v>
       </c>
     </row>
     <row r="55">
@@ -3896,62 +3896,62 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>31/03/2024</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Nacional de Potosí</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K55" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L55" t="n">
         <v>5</v>
       </c>
       <c r="M55" t="n">
+        <v>2</v>
+      </c>
+      <c r="N55" t="n">
         <v>1</v>
       </c>
-      <c r="N55" t="n">
-        <v>4</v>
-      </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P55" t="n">
-        <v>2.9611</v>
+        <v>2.9749</v>
       </c>
     </row>
     <row r="56">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>27/01/2024</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3973,17 +3973,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -4001,21 +4001,21 @@
         <v>5</v>
       </c>
       <c r="L56" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M56" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2.9303</v>
+        <v>2.9682</v>
       </c>
     </row>
     <row r="57">
@@ -4024,11 +4024,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>11/01/2025</t>
+          <t>31/03/2024</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -4037,22 +4037,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Maricá</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -4062,10 +4062,10 @@
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L57" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M57" t="n">
         <v>1</v>
@@ -4079,7 +4079,7 @@
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.9303</v>
+        <v>2.9611</v>
       </c>
     </row>
     <row r="58">
@@ -4088,25 +4088,25 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>27/01/2024</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -4116,34 +4116,34 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J58" t="n">
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L58" t="n">
         <v>3</v>
       </c>
       <c r="M58" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2.8806</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="59">
@@ -4152,11 +4152,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>11/01/2025</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -4165,22 +4165,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Maricá</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -4190,10 +4190,10 @@
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M59" t="n">
         <v>1</v>
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2.861</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="60">
@@ -4216,11 +4216,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>18/08/2024</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -4234,44 +4234,44 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I60" t="n">
         <v>4</v>
       </c>
       <c r="J60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K60" t="n">
         <v>3</v>
       </c>
       <c r="L60" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M60" t="n">
         <v>4</v>
       </c>
       <c r="N60" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2.7651</v>
+        <v>2.8806</v>
       </c>
     </row>
     <row r="61">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>24/01/2026</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -4293,22 +4293,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -4321,7 +4321,7 @@
         <v>3</v>
       </c>
       <c r="L61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M61" t="n">
         <v>1</v>
@@ -4335,7 +4335,7 @@
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2.7609</v>
+        <v>2.861</v>
       </c>
     </row>
     <row r="62">
@@ -4344,62 +4344,62 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>SEMIS - TR</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" t="n">
         <v>3</v>
       </c>
       <c r="L62" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M62" t="n">
+        <v>4</v>
+      </c>
+      <c r="N62" t="n">
         <v>1</v>
       </c>
-      <c r="N62" t="n">
-        <v>4</v>
-      </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P62" t="n">
-        <v>2.7609</v>
+        <v>2.7651</v>
       </c>
     </row>
     <row r="63">
@@ -4408,62 +4408,62 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>29/07/2025</t>
+          <t>24/01/2026</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K63" t="n">
         <v>3</v>
       </c>
       <c r="L63" t="n">
+        <v>3</v>
+      </c>
+      <c r="M63" t="n">
         <v>1</v>
       </c>
-      <c r="M63" t="n">
-        <v>2</v>
-      </c>
       <c r="N63" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P63" t="n">
-        <v>2.7495</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="64">
@@ -4472,39 +4472,39 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>SEMIS - TR</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J64" t="n">
         <v>2</v>
@@ -4513,21 +4513,21 @@
         <v>3</v>
       </c>
       <c r="L64" t="n">
+        <v>3</v>
+      </c>
+      <c r="M64" t="n">
         <v>1</v>
       </c>
-      <c r="M64" t="n">
-        <v>2</v>
-      </c>
       <c r="N64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P64" t="n">
-        <v>2.7208</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="65">

</xml_diff>

<commit_message>
AHP: adiciona Recopa Sulamericana ao grupo de competições noturnas
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -2040,62 +2040,62 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>17/03/2024</t>
+          <t>27/02/2025</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Recopa</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Racing</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>FINAL</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J26" t="n">
         <v>5</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M26" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" t="n">
         <v>1</v>
       </c>
-      <c r="N26" t="n">
-        <v>3</v>
-      </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>3.58</v>
+        <v>3.5968</v>
       </c>
     </row>
     <row r="27">
@@ -2104,62 +2104,62 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>17/03/2024</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K27" t="n">
         <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>3.5543</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="28">
@@ -2168,45 +2168,45 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J28" t="n">
         <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L28" t="n">
         <v>4</v>
@@ -2215,15 +2215,15 @@
         <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.5515</v>
+        <v>3.5543</v>
       </c>
     </row>
     <row r="29">
@@ -2232,25 +2232,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2264,30 +2264,30 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.5303</v>
+        <v>3.5515</v>
       </c>
     </row>
     <row r="30">
@@ -2296,11 +2296,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2309,35 +2309,35 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I30" t="n">
         <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
         <v>4</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>3.5045</v>
+        <v>3.5303</v>
       </c>
     </row>
     <row r="31">
@@ -2360,11 +2360,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>23/11/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2388,14 +2388,14 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I31" t="n">
         <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
@@ -2404,18 +2404,18 @@
         <v>3</v>
       </c>
       <c r="M31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>3.4517</v>
+        <v>3.5045</v>
       </c>
     </row>
     <row r="32">
@@ -2424,62 +2424,62 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>23/11/2024</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K32" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>3.4252</v>
+        <v>3.4517</v>
       </c>
     </row>
     <row r="33">
@@ -2488,62 +2488,62 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M33" t="n">
         <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.4198</v>
+        <v>3.4252</v>
       </c>
     </row>
     <row r="34">
@@ -2552,62 +2552,62 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J34" t="n">
         <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.4128</v>
+        <v>3.4198</v>
       </c>
     </row>
     <row r="35">
@@ -2616,30 +2616,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2657,10 +2657,10 @@
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
         <v>4</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.363</v>
+        <v>3.4128</v>
       </c>
     </row>
     <row r="36">
@@ -2680,51 +2680,51 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.3437</v>
+        <v>3.363</v>
       </c>
     </row>
     <row r="37">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2757,22 +2757,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -2785,10 +2785,10 @@
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N37" t="n">
         <v>4</v>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.2939</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="38">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2816,37 +2816,37 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J38" t="n">
         <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L38" t="n">
         <v>4</v>
@@ -2855,15 +2855,15 @@
         <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.2911</v>
+        <v>3.2939</v>
       </c>
     </row>
     <row r="39">
@@ -2872,25 +2872,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2904,10 +2904,10 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K39" t="n">
         <v>5</v>
@@ -2916,7 +2916,7 @@
         <v>4</v>
       </c>
       <c r="M39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N39" t="n">
         <v>3</v>
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2695</v>
+        <v>3.2911</v>
       </c>
     </row>
     <row r="40">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2944,40 +2944,40 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M40" t="n">
         <v>3</v>
@@ -2987,11 +2987,11 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2515</v>
+        <v>3.2695</v>
       </c>
     </row>
     <row r="41">
@@ -3000,11 +3000,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>18/10/2024</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3013,22 +3013,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Criciúma</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sexta-feira</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3077,22 +3077,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -3102,24 +3102,24 @@
         <v>4</v>
       </c>
       <c r="K42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2452</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="43">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/02/2025</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -3136,40 +3136,40 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Recopa</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Racing</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>FINAL</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L43" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M43" t="n">
         <v>4</v>
@@ -3179,11 +3179,11 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.2426</v>
+        <v>3.2452</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
AHP: limita score de fase a 2 para Carioca / Taça Rio
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -2104,62 +2104,62 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>17/03/2024</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
         <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>3.58</v>
+        <v>3.5543</v>
       </c>
     </row>
     <row r="28">
@@ -2168,45 +2168,45 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J28" t="n">
         <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L28" t="n">
         <v>4</v>
@@ -2215,15 +2215,15 @@
         <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.5543</v>
+        <v>3.5515</v>
       </c>
     </row>
     <row r="29">
@@ -2232,25 +2232,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2264,30 +2264,30 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.5515</v>
+        <v>3.5303</v>
       </c>
     </row>
     <row r="30">
@@ -2296,11 +2296,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2309,35 +2309,35 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I30" t="n">
         <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M30" t="n">
         <v>4</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>3.5303</v>
+        <v>3.5045</v>
       </c>
     </row>
     <row r="31">
@@ -2360,11 +2360,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>23/11/2024</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2388,14 +2388,14 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I31" t="n">
         <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
@@ -2404,18 +2404,18 @@
         <v>3</v>
       </c>
       <c r="M31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>3.5045</v>
+        <v>3.4517</v>
       </c>
     </row>
     <row r="32">
@@ -2424,62 +2424,62 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23/11/2024</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K32" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>3.4517</v>
+        <v>3.4252</v>
       </c>
     </row>
     <row r="33">
@@ -2488,62 +2488,62 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
         <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.4252</v>
+        <v>3.4198</v>
       </c>
     </row>
     <row r="34">
@@ -2552,62 +2552,62 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
         <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.4198</v>
+        <v>3.4128</v>
       </c>
     </row>
     <row r="35">
@@ -2616,30 +2616,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2657,10 +2657,10 @@
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
         <v>4</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.4128</v>
+        <v>3.363</v>
       </c>
     </row>
     <row r="36">
@@ -2680,51 +2680,51 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.363</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="37">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2757,22 +2757,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -2785,10 +2785,10 @@
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N37" t="n">
         <v>4</v>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.3437</v>
+        <v>3.2939</v>
       </c>
     </row>
     <row r="38">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2816,37 +2816,37 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J38" t="n">
         <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L38" t="n">
         <v>4</v>
@@ -2855,15 +2855,15 @@
         <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.2939</v>
+        <v>3.2911</v>
       </c>
     </row>
     <row r="39">
@@ -2872,25 +2872,25 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2904,10 +2904,10 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K39" t="n">
         <v>5</v>
@@ -2916,7 +2916,7 @@
         <v>4</v>
       </c>
       <c r="M39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N39" t="n">
         <v>3</v>
@@ -2927,7 +2927,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2911</v>
+        <v>3.2695</v>
       </c>
     </row>
     <row r="40">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>18/10/2024</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2944,40 +2944,40 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Criciúma</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sexta-feira</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
         <v>3</v>
@@ -2987,11 +2987,11 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2695</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="41">
@@ -3000,11 +3000,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3013,22 +3013,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3077,22 +3077,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -3102,24 +3102,24 @@
         <v>4</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
+        <v>5</v>
+      </c>
+      <c r="M42" t="n">
+        <v>4</v>
+      </c>
+      <c r="N42" t="n">
         <v>1</v>
       </c>
-      <c r="M42" t="n">
-        <v>3</v>
-      </c>
-      <c r="N42" t="n">
-        <v>3</v>
-      </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2515</v>
+        <v>3.2452</v>
       </c>
     </row>
     <row r="43">
@@ -3128,11 +3128,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>14/09/2024</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -3141,49 +3141,49 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I43" t="n">
         <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M43" t="n">
         <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.2452</v>
+        <v>3.1913</v>
       </c>
     </row>
     <row r="44">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>14/09/2024</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -3205,22 +3205,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -3233,21 +3233,21 @@
         <v>3</v>
       </c>
       <c r="L44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
         <v>3</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>3.1913</v>
+        <v>3.1908</v>
       </c>
     </row>
     <row r="45">
@@ -3256,11 +3256,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>17/09/2025</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>17/09/2025</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3333,12 +3333,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -3358,13 +3358,13 @@
         <v>3</v>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L46" t="n">
         <v>4</v>
       </c>
       <c r="M46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N46" t="n">
         <v>3</v>
@@ -3375,7 +3375,7 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.1908</v>
+        <v>3.1564</v>
       </c>
     </row>
     <row r="47">
@@ -3384,11 +3384,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>31/08/2024</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3397,22 +3397,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -3422,10 +3422,10 @@
         <v>3</v>
       </c>
       <c r="K47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M47" t="n">
         <v>3</v>
@@ -3435,11 +3435,11 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>3.1564</v>
+        <v>3.141</v>
       </c>
     </row>
     <row r="48">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>31/08/2024</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3461,49 +3461,49 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I48" t="n">
         <v>4</v>
       </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
       </c>
       <c r="M48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>3.141</v>
+        <v>3.1091</v>
       </c>
     </row>
     <row r="49">
@@ -3512,11 +3512,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3525,49 +3525,49 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I49" t="n">
         <v>4</v>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L49" t="n">
         <v>3</v>
       </c>
       <c r="M49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>3.1091</v>
+        <v>3.0907</v>
       </c>
     </row>
     <row r="50">
@@ -3576,62 +3576,62 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J50" t="n">
         <v>3</v>
       </c>
       <c r="K50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>3.0907</v>
+        <v>3.0755</v>
       </c>
     </row>
     <row r="51">
@@ -3640,20 +3640,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>29/07/2025</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3663,39 +3663,39 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J51" t="n">
         <v>3</v>
       </c>
       <c r="K51" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>3.0755</v>
+        <v>3.0498</v>
       </c>
     </row>
     <row r="52">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>29/07/2025</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3712,17 +3712,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3736,10 +3736,10 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="n">
         <v>3</v>
@@ -3755,11 +3755,11 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>3.0498</v>
+        <v>3.0211</v>
       </c>
     </row>
     <row r="53">
@@ -3768,25 +3768,25 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3796,11 +3796,11 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J53" t="n">
         <v>2</v>
@@ -3809,21 +3809,21 @@
         <v>3</v>
       </c>
       <c r="L53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P53" t="n">
-        <v>3.0211</v>
+        <v>2.9936</v>
       </c>
     </row>
     <row r="54">
@@ -3832,62 +3832,62 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Nacional de Potosí</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I54" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K54" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L54" t="n">
+        <v>5</v>
+      </c>
+      <c r="M54" t="n">
+        <v>2</v>
+      </c>
+      <c r="N54" t="n">
         <v>1</v>
       </c>
-      <c r="M54" t="n">
-        <v>4</v>
-      </c>
-      <c r="N54" t="n">
-        <v>4</v>
-      </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2.9936</v>
+        <v>2.9749</v>
       </c>
     </row>
     <row r="55">
@@ -3896,42 +3896,42 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Nacional de Potosí</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
         <v>5</v>
@@ -3940,18 +3940,18 @@
         <v>5</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N55" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P55" t="n">
-        <v>2.9749</v>
+        <v>2.9682</v>
       </c>
     </row>
     <row r="56">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>31/03/2024</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -3998,24 +3998,24 @@
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L56" t="n">
         <v>5</v>
       </c>
       <c r="M56" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2.9682</v>
+        <v>2.9611</v>
       </c>
     </row>
     <row r="57">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>31/03/2024</t>
+          <t>27/01/2024</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4037,22 +4037,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -4062,10 +4062,10 @@
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L57" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M57" t="n">
         <v>1</v>
@@ -4079,7 +4079,7 @@
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.9611</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="58">
@@ -4088,11 +4088,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>27/01/2024</t>
+          <t>11/01/2025</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -4101,12 +4101,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Maricá</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -4152,25 +4152,25 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>11/01/2025</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Maricá</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4180,34 +4180,34 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L59" t="n">
         <v>3</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2.9303</v>
+        <v>2.8806</v>
       </c>
     </row>
     <row r="60">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -4224,31 +4224,31 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J60" t="n">
         <v>2</v>
@@ -4257,21 +4257,21 @@
         <v>3</v>
       </c>
       <c r="L60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M60" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2.8806</v>
+        <v>2.861</v>
       </c>
     </row>
     <row r="61">
@@ -4280,62 +4280,62 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K61" t="n">
         <v>3</v>
       </c>
       <c r="L61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M61" t="n">
+        <v>4</v>
+      </c>
+      <c r="N61" t="n">
         <v>1</v>
       </c>
-      <c r="N61" t="n">
-        <v>4</v>
-      </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2.861</v>
+        <v>2.7651</v>
       </c>
     </row>
     <row r="62">
@@ -4344,62 +4344,62 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>18/08/2024</t>
+          <t>24/01/2026</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="n">
         <v>3</v>
       </c>
       <c r="L62" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M62" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P62" t="n">
-        <v>2.7651</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="63">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>24/01/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -4421,12 +4421,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>SEMIS - TR</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I63" t="n">
@@ -4472,30 +4472,30 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>15/10/2025</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>SEMIS - TR</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4504,30 +4504,30 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K64" t="n">
         <v>3</v>
       </c>
       <c r="L64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M64" t="n">
+        <v>4</v>
+      </c>
+      <c r="N64" t="n">
         <v>1</v>
       </c>
-      <c r="N64" t="n">
-        <v>4</v>
-      </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P64" t="n">
-        <v>2.7609</v>
+        <v>2.665</v>
       </c>
     </row>
     <row r="65">
@@ -4536,62 +4536,62 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>15/10/2025</t>
+          <t>17/03/2024</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K65" t="n">
         <v>3</v>
       </c>
       <c r="L65" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M65" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P65" t="n">
-        <v>2.665</v>
+        <v>2.6479</v>
       </c>
     </row>
     <row r="66">
@@ -4600,62 +4600,62 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15/02/2026</t>
+          <t>16/07/2025</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Quartas</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>D+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P66" t="n">
-        <v>2.5653</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="67">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>16/07/2025</t>
+          <t>20/09/2025</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -4677,22 +4677,22 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -4702,10 +4702,10 @@
         <v>3</v>
       </c>
       <c r="K67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M67" t="n">
         <v>3</v>
@@ -4715,11 +4715,11 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+E+D</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>2.53</v>
+        <v>2.5146</v>
       </c>
     </row>
     <row r="68">
@@ -4728,62 +4728,62 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>20/09/2025</t>
+          <t>30/01/2024</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Portuguesa</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N68" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>E+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P68" t="n">
-        <v>2.5146</v>
+        <v>2.476</v>
       </c>
     </row>
     <row r="69">
@@ -4792,11 +4792,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>30/01/2024</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -4805,22 +4805,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Portuguesa</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>FINAL - TR</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -4830,24 +4830,24 @@
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M69" t="n">
         <v>1</v>
       </c>
       <c r="N69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P69" t="n">
-        <v>2.476</v>
+        <v>2.4477</v>
       </c>
     </row>
     <row r="70">
@@ -4856,39 +4856,39 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>21/04/2024</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>FINAL - TR</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J70" t="n">
         <v>2</v>
@@ -4897,21 +4897,21 @@
         <v>3</v>
       </c>
       <c r="L70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M70" t="n">
+        <v>2</v>
+      </c>
+      <c r="N70" t="n">
         <v>1</v>
       </c>
-      <c r="N70" t="n">
-        <v>3</v>
-      </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P70" t="n">
-        <v>2.4477</v>
+        <v>2.3538</v>
       </c>
     </row>
     <row r="71">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>21/04/2024</t>
+          <t>26/04/2025</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -4933,22 +4933,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I71" t="n">
@@ -4961,21 +4961,21 @@
         <v>3</v>
       </c>
       <c r="L71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M71" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N71" t="n">
         <v>1</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P71" t="n">
-        <v>2.3538</v>
+        <v>2.2542</v>
       </c>
     </row>
     <row r="72">
@@ -4984,11 +4984,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -4997,22 +4997,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -5025,21 +5025,21 @@
         <v>3</v>
       </c>
       <c r="L72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M72" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N72" t="n">
         <v>1</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P72" t="n">
-        <v>2.2542</v>
+        <v>2.2537</v>
       </c>
     </row>
     <row r="73">
@@ -5048,11 +5048,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>05/04/2025</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -5061,22 +5061,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -5089,7 +5089,7 @@
         <v>3</v>
       </c>
       <c r="L73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M73" t="n">
         <v>2</v>
@@ -5099,11 +5099,11 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>2.2537</v>
+        <v>2.1536</v>
       </c>
     </row>
     <row r="74">
@@ -5112,11 +5112,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>05/04/2025</t>
+          <t>18/04/2024</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Atlético-GO</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5135,12 +5135,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I74" t="n">
@@ -5150,7 +5150,7 @@
         <v>2</v>
       </c>
       <c r="K74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L74" t="n">
         <v>3</v>
@@ -5163,11 +5163,11 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P74" t="n">
-        <v>2.1536</v>
+        <v>2.0689</v>
       </c>
     </row>
     <row r="75">
@@ -5176,51 +5176,51 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>18/04/2024</t>
+          <t>26/01/2025</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Atlético-GO</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I75" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J75" t="n">
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L75" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N75" t="n">
         <v>1</v>
@@ -5231,7 +5231,7 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>2.0689</v>
+        <v>2.0215</v>
       </c>
     </row>
     <row r="76">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>26/01/2025</t>
+          <t>29/01/2025</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -5253,22 +5253,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -5278,13 +5278,13 @@
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N76" t="n">
         <v>1</v>
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>2.0215</v>
+        <v>1.9876</v>
       </c>
     </row>
     <row r="77">
@@ -5304,11 +5304,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>29/01/2025</t>
+          <t>15/02/2026</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -5317,22 +5317,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Quartas</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -5342,24 +5342,24 @@
         <v>2</v>
       </c>
       <c r="K77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M77" t="n">
         <v>4</v>
       </c>
       <c r="N77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>D+D+D</t>
         </is>
       </c>
       <c r="P77" t="n">
-        <v>1.9876</v>
+        <v>1.9439</v>
       </c>
     </row>
     <row r="78">

</xml_diff>

<commit_message>
Update dPartidas.xlsx from colleague's branch and regenerate data
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -952,11 +952,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>08/05/2024</t>
+          <t>14/05/2025</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -965,7 +965,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Estudiantes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -996,7 +996,7 @@
         <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" t="n">
         <v>4</v>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>3.9648</v>
+        <v>4.0151</v>
       </c>
     </row>
     <row r="10">
@@ -1016,30 +1016,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11/09/2025</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1048,30 +1048,30 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N10" t="n">
         <v>4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>3.9437</v>
+        <v>3.9648</v>
       </c>
     </row>
     <row r="11">
@@ -1080,39 +1080,39 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>11/09/2025</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>QUARTAS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
         <v>4</v>
@@ -1121,21 +1121,21 @@
         <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" t="n">
         <v>4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>3.9343</v>
+        <v>3.9437</v>
       </c>
     </row>
     <row r="12">
@@ -1144,11 +1144,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>03/08/2025</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1157,49 +1157,49 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I12" t="n">
         <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
         <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12" t="n">
         <v>4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.8741</v>
+        <v>3.9343</v>
       </c>
     </row>
     <row r="13">
@@ -1208,11 +1208,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>19/06/2024</t>
+          <t>03/08/2025</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1221,22 +1221,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Athlético</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1246,24 +1246,24 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>3.8675</v>
+        <v>3.8741</v>
       </c>
     </row>
     <row r="14">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>17/07/2024</t>
+          <t>19/06/2024</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1285,12 +1285,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Athlético</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1310,13 +1310,13 @@
         <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" t="n">
         <v>4</v>
       </c>
       <c r="M14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" t="n">
         <v>5</v>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>3.8331</v>
+        <v>3.8675</v>
       </c>
     </row>
     <row r="15">
@@ -1336,11 +1336,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>17/07/2024</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1349,22 +1349,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1374,24 +1374,24 @@
         <v>3</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>3.8238</v>
+        <v>3.8331</v>
       </c>
     </row>
     <row r="16">
@@ -1400,45 +1400,45 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Universitario</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
         <v>5</v>
@@ -1451,11 +1451,11 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>3.7954</v>
+        <v>3.8238</v>
       </c>
     </row>
     <row r="17">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>20/07/2024</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1472,31 +1472,31 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Universitario</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J17" t="n">
         <v>3</v>
@@ -1505,21 +1505,21 @@
         <v>3</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M17" t="n">
         <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>3.7674</v>
+        <v>3.7954</v>
       </c>
     </row>
     <row r="18">
@@ -1528,11 +1528,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>22/11/2025</t>
+          <t>20/07/2024</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Grêmio</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1556,14 +1556,14 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I18" t="n">
         <v>4</v>
       </c>
       <c r="J18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K18" t="n">
         <v>3</v>
@@ -1575,15 +1575,15 @@
         <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>3.7649</v>
+        <v>3.7674</v>
       </c>
     </row>
     <row r="19">
@@ -1592,62 +1592,62 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>22/11/2025</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Grêmio</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K19" t="n">
         <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M19" t="n">
         <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>3.7265</v>
+        <v>3.7649</v>
       </c>
     </row>
     <row r="20">
@@ -1656,62 +1656,62 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>14/05/2025</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Estudiantes</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>3.7044</v>
+        <v>3.7265</v>
       </c>
     </row>
     <row r="21">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1989,17 +1989,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aurora</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2017,10 +2017,10 @@
         <v>5</v>
       </c>
       <c r="L25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N25" t="n">
         <v>3</v>
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>3.6013</v>
+        <v>3.6018</v>
       </c>
     </row>
     <row r="26">
@@ -2040,30 +2040,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>27/02/2025</t>
+          <t>28/02/2024</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Recopa</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Racing</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>FINAL</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2075,27 +2075,27 @@
         <v>5</v>
       </c>
       <c r="J26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K26" t="n">
         <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>3.5968</v>
+        <v>3.6013</v>
       </c>
     </row>
     <row r="27">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>27/02/2025</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -2112,54 +2112,54 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Recopa</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Racing</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>FINAL</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L27" t="n">
         <v>4</v>
       </c>
       <c r="M27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>3.5543</v>
+        <v>3.5968</v>
       </c>
     </row>
     <row r="28">
@@ -2168,45 +2168,45 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J28" t="n">
         <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L28" t="n">
         <v>4</v>
@@ -2215,15 +2215,15 @@
         <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.5515</v>
+        <v>3.5543</v>
       </c>
     </row>
     <row r="29">
@@ -2232,25 +2232,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2264,30 +2264,30 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.5303</v>
+        <v>3.5515</v>
       </c>
     </row>
     <row r="30">
@@ -2296,11 +2296,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2309,35 +2309,35 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I30" t="n">
         <v>4</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
         <v>4</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>3.5045</v>
+        <v>3.5303</v>
       </c>
     </row>
     <row r="31">
@@ -2360,11 +2360,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>23/11/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2388,14 +2388,14 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I31" t="n">
         <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
@@ -2404,18 +2404,18 @@
         <v>3</v>
       </c>
       <c r="M31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>3.4517</v>
+        <v>3.5045</v>
       </c>
     </row>
     <row r="32">
@@ -2424,62 +2424,62 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>23/11/2024</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K32" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N32" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>3.4252</v>
+        <v>3.4517</v>
       </c>
     </row>
     <row r="33">
@@ -2488,62 +2488,62 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M33" t="n">
         <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.4198</v>
+        <v>3.4252</v>
       </c>
     </row>
     <row r="34">
@@ -2552,62 +2552,62 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J34" t="n">
         <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.4128</v>
+        <v>3.4198</v>
       </c>
     </row>
     <row r="35">
@@ -2616,30 +2616,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2657,10 +2657,10 @@
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
         <v>4</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.363</v>
+        <v>3.4128</v>
       </c>
     </row>
     <row r="36">
@@ -2680,51 +2680,51 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.3437</v>
+        <v>3.363</v>
       </c>
     </row>
     <row r="37">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2757,22 +2757,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -2785,10 +2785,10 @@
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N37" t="n">
         <v>4</v>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.2939</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="38">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2821,12 +2821,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2836,23 +2836,23 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I38" t="n">
         <v>5</v>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K38" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L38" t="n">
         <v>4</v>
       </c>
       <c r="M38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N38" t="n">
         <v>3</v>
@@ -2863,7 +2863,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.2911</v>
+        <v>3.3318</v>
       </c>
     </row>
     <row r="39">
@@ -2872,62 +2872,62 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L39" t="n">
         <v>4</v>
       </c>
       <c r="M39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2695</v>
+        <v>3.2939</v>
       </c>
     </row>
     <row r="40">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2944,40 +2944,40 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M40" t="n">
         <v>3</v>
@@ -2987,11 +2987,11 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2515</v>
+        <v>3.2695</v>
       </c>
     </row>
     <row r="41">
@@ -3000,11 +3000,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>18/10/2024</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3013,22 +3013,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Criciúma</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sexta-feira</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3077,22 +3077,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -3102,24 +3102,24 @@
         <v>4</v>
       </c>
       <c r="K42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2452</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="43">
@@ -3128,11 +3128,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>14/09/2024</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -3141,49 +3141,49 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I43" t="n">
         <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K43" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L43" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M43" t="n">
         <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.1913</v>
+        <v>3.2452</v>
       </c>
     </row>
     <row r="44">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>14/09/2024</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -3205,22 +3205,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -3233,21 +3233,21 @@
         <v>3</v>
       </c>
       <c r="L44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N44" t="n">
         <v>3</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>3.1908</v>
+        <v>3.1913</v>
       </c>
     </row>
     <row r="45">
@@ -3256,11 +3256,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>17/09/2025</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>17/09/2025</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3333,12 +3333,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -3358,13 +3358,13 @@
         <v>3</v>
       </c>
       <c r="K46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L46" t="n">
         <v>4</v>
       </c>
       <c r="M46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N46" t="n">
         <v>3</v>
@@ -3375,7 +3375,7 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.1564</v>
+        <v>3.1908</v>
       </c>
     </row>
     <row r="47">
@@ -3384,11 +3384,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>31/08/2024</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -3397,22 +3397,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -3422,10 +3422,10 @@
         <v>3</v>
       </c>
       <c r="K47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M47" t="n">
         <v>3</v>
@@ -3435,11 +3435,11 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>3.141</v>
+        <v>3.1564</v>
       </c>
     </row>
     <row r="48">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>31/08/2024</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3461,49 +3461,49 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I48" t="n">
         <v>4</v>
       </c>
       <c r="J48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>3.1091</v>
+        <v>3.141</v>
       </c>
     </row>
     <row r="49">
@@ -3512,11 +3512,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3525,49 +3525,49 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I49" t="n">
         <v>4</v>
       </c>
       <c r="J49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L49" t="n">
         <v>3</v>
       </c>
       <c r="M49" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>3.0907</v>
+        <v>3.1091</v>
       </c>
     </row>
     <row r="50">
@@ -3576,62 +3576,62 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J50" t="n">
         <v>3</v>
       </c>
       <c r="K50" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M50" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>3.0755</v>
+        <v>3.0907</v>
       </c>
     </row>
     <row r="51">
@@ -3640,20 +3640,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>29/07/2025</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3663,39 +3663,39 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J51" t="n">
         <v>3</v>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L51" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>3.0498</v>
+        <v>3.0755</v>
       </c>
     </row>
     <row r="52">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>29/07/2025</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3712,17 +3712,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3736,10 +3736,10 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="n">
         <v>3</v>
@@ -3755,11 +3755,11 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>3.0211</v>
+        <v>3.0498</v>
       </c>
     </row>
     <row r="53">

</xml_diff>

<commit_message>
AHP: limita score de dia da semana a 3 para Carioca
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -2488,62 +2488,62 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
         <v>4</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.4252</v>
+        <v>3.4198</v>
       </c>
     </row>
     <row r="34">
@@ -2552,62 +2552,62 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
         <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
         <v>4</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.4198</v>
+        <v>3.4128</v>
       </c>
     </row>
     <row r="35">
@@ -2616,30 +2616,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2657,10 +2657,10 @@
         <v>3</v>
       </c>
       <c r="L35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
         <v>4</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.4128</v>
+        <v>3.363</v>
       </c>
     </row>
     <row r="36">
@@ -2680,51 +2680,51 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.363</v>
+        <v>3.3437</v>
       </c>
     </row>
     <row r="37">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -2752,54 +2752,54 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K37" t="n">
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.3437</v>
+        <v>3.3318</v>
       </c>
     </row>
     <row r="38">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2816,34 +2816,34 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
         <v>3</v>
@@ -2852,18 +2852,18 @@
         <v>4</v>
       </c>
       <c r="M38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.3318</v>
+        <v>3.2939</v>
       </c>
     </row>
     <row r="39">
@@ -2872,62 +2872,62 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L39" t="n">
         <v>4</v>
       </c>
       <c r="M39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2939</v>
+        <v>3.2695</v>
       </c>
     </row>
     <row r="40">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>18/10/2024</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2944,40 +2944,40 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Criciúma</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sexta-feira</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
         <v>3</v>
@@ -2987,11 +2987,11 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2695</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="41">
@@ -3000,11 +3000,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3013,22 +3013,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3077,22 +3077,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -3102,24 +3102,24 @@
         <v>4</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
+        <v>5</v>
+      </c>
+      <c r="M42" t="n">
+        <v>4</v>
+      </c>
+      <c r="N42" t="n">
         <v>1</v>
       </c>
-      <c r="M42" t="n">
-        <v>3</v>
-      </c>
-      <c r="N42" t="n">
-        <v>3</v>
-      </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2515</v>
+        <v>3.2452</v>
       </c>
     </row>
     <row r="43">
@@ -3128,25 +3128,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3156,34 +3156,34 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M43" t="n">
         <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.2452</v>
+        <v>3.225</v>
       </c>
     </row>
     <row r="44">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>27/01/2024</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3909,17 +3909,17 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3937,21 +3937,21 @@
         <v>5</v>
       </c>
       <c r="L55" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M55" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P55" t="n">
-        <v>2.9682</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="56">
@@ -3960,11 +3960,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>31/03/2024</t>
+          <t>11/01/2025</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -3973,22 +3973,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Maricá</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -3998,10 +3998,10 @@
         <v>2</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L56" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M56" t="n">
         <v>1</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2.9611</v>
+        <v>2.9303</v>
       </c>
     </row>
     <row r="57">
@@ -4024,25 +4024,25 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>27/01/2024</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4052,34 +4052,34 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J57" t="n">
         <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L57" t="n">
         <v>3</v>
       </c>
       <c r="M57" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.9303</v>
+        <v>2.8806</v>
       </c>
     </row>
     <row r="58">
@@ -4088,11 +4088,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>11/01/2025</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -4101,17 +4101,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Maricá</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4132,18 +4132,18 @@
         <v>3</v>
       </c>
       <c r="M58" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2.9303</v>
+        <v>2.768</v>
       </c>
     </row>
     <row r="59">
@@ -4152,11 +4152,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -4170,44 +4170,44 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I59" t="n">
         <v>4</v>
       </c>
       <c r="J59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="n">
         <v>3</v>
       </c>
       <c r="L59" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M59" t="n">
         <v>4</v>
       </c>
       <c r="N59" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2.8806</v>
+        <v>2.7651</v>
       </c>
     </row>
     <row r="60">
@@ -4216,11 +4216,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>31/03/2024</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -4229,22 +4229,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -4257,7 +4257,7 @@
         <v>3</v>
       </c>
       <c r="L60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M60" t="n">
         <v>1</v>
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2.861</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="61">
@@ -4280,62 +4280,62 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>18/08/2024</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K61" t="n">
         <v>3</v>
       </c>
       <c r="L61" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M61" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N61" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2.7651</v>
+        <v>2.7609</v>
       </c>
     </row>
     <row r="62">
@@ -4536,62 +4536,62 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>17/03/2024</t>
+          <t>16/07/2025</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M65" t="n">
+        <v>3</v>
+      </c>
+      <c r="N65" t="n">
         <v>1</v>
       </c>
-      <c r="N65" t="n">
-        <v>3</v>
-      </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P65" t="n">
-        <v>2.6479</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="66">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>16/07/2025</t>
+          <t>20/09/2025</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -4613,22 +4613,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I66" t="n">
@@ -4638,10 +4638,10 @@
         <v>3</v>
       </c>
       <c r="K66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M66" t="n">
         <v>3</v>
@@ -4651,11 +4651,11 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+E+D</t>
         </is>
       </c>
       <c r="P66" t="n">
-        <v>2.53</v>
+        <v>2.5146</v>
       </c>
     </row>
     <row r="67">
@@ -4664,62 +4664,62 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>20/09/2025</t>
+          <t>30/01/2024</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Portuguesa</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M67" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N67" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>E+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>2.5146</v>
+        <v>2.476</v>
       </c>
     </row>
     <row r="68">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>30/01/2024</t>
+          <t>17/03/2024</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -4741,22 +4741,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Portuguesa</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -4766,24 +4766,24 @@
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M68" t="n">
         <v>1</v>
       </c>
       <c r="N68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P68" t="n">
-        <v>2.476</v>
+        <v>2.4477</v>
       </c>
     </row>
     <row r="69">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>26/01/2025</t>
+          <t>29/01/2025</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -5189,22 +5189,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -5214,13 +5214,13 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L75" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N75" t="n">
         <v>1</v>
@@ -5231,7 +5231,7 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>2.0215</v>
+        <v>1.8875</v>
       </c>
     </row>
     <row r="76">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>29/01/2025</t>
+          <t>26/01/2025</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -5253,22 +5253,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -5278,13 +5278,13 @@
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N76" t="n">
         <v>1</v>
@@ -5295,7 +5295,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>1.9876</v>
+        <v>1.8213</v>
       </c>
     </row>
     <row r="77">
@@ -5345,7 +5345,7 @@
         <v>4</v>
       </c>
       <c r="L77" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M77" t="n">
         <v>4</v>
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>1.9439</v>
+        <v>1.7437</v>
       </c>
     </row>
     <row r="78">
@@ -5409,7 +5409,7 @@
         <v>2</v>
       </c>
       <c r="L78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M78" t="n">
         <v>1</v>
@@ -5423,7 +5423,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>1.8367</v>
+        <v>1.7366</v>
       </c>
     </row>
     <row r="79">
@@ -5537,7 +5537,7 @@
         <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M80" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
AHP: exclui Criciúma 2024 da análise (outlier — jogo decisivo pelo título)
Pearson r: 0.767 → 0.806 | Spearman r: 0.803 → 0.817

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P81"/>
+  <dimension ref="A1:P80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2424,11 +2424,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>18/10/2024</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Criciúma</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sexta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I32" t="n">
@@ -2488,11 +2488,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>20/07/2024</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2501,49 +2501,49 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I33" t="n">
         <v>4</v>
       </c>
       <c r="J33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K33" t="n">
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
         <v>3</v>
       </c>
       <c r="N33" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.3345</v>
+        <v>3.3235</v>
       </c>
     </row>
     <row r="34">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>20/07/2024</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2560,54 +2560,54 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L34" t="n">
         <v>3</v>
       </c>
       <c r="M34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.3235</v>
+        <v>3.308</v>
       </c>
     </row>
     <row r="35">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2624,37 +2624,37 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L35" t="n">
         <v>3</v>
@@ -2663,15 +2663,15 @@
         <v>4</v>
       </c>
       <c r="N35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.308</v>
+        <v>3.3016</v>
       </c>
     </row>
     <row r="36">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>07/07/2024</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2693,22 +2693,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -2718,13 +2718,13 @@
         <v>3</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.3016</v>
+        <v>3.2777</v>
       </c>
     </row>
     <row r="37">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07/07/2024</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2757,49 +2757,49 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I37" t="n">
         <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K37" t="n">
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N37" t="n">
         <v>4</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.2777</v>
+        <v>3.2742</v>
       </c>
     </row>
     <row r="38">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2821,17 +2821,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2843,27 +2843,27 @@
         <v>4</v>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K38" t="n">
         <v>3</v>
       </c>
       <c r="L38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M38" t="n">
         <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.2742</v>
+        <v>3.2656</v>
       </c>
     </row>
     <row r="39">
@@ -2872,11 +2872,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18/08/2024</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2885,22 +2885,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -2913,21 +2913,21 @@
         <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2656</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="40">
@@ -2936,25 +2936,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Nacional de Potosí</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2964,34 +2964,34 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J40" t="n">
         <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2515</v>
+        <v>3.2401</v>
       </c>
     </row>
     <row r="41">
@@ -3000,25 +3000,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>15/10/2025</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Nacional de Potosí</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3028,23 +3028,23 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
         <v>3</v>
       </c>
       <c r="K41" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N41" t="n">
         <v>1</v>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>3.2401</v>
+        <v>3.2394</v>
       </c>
     </row>
     <row r="42">
@@ -3064,39 +3064,39 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>15/10/2025</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J42" t="n">
         <v>3</v>
@@ -3108,18 +3108,18 @@
         <v>4</v>
       </c>
       <c r="M42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2394</v>
+        <v>3.2226</v>
       </c>
     </row>
     <row r="43">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -3136,54 +3136,54 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K43" t="n">
         <v>3</v>
       </c>
       <c r="L43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.2226</v>
+        <v>3.1956</v>
       </c>
     </row>
     <row r="44">
@@ -3192,11 +3192,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3205,22 +3205,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -3233,21 +3233,21 @@
         <v>3</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M44" t="n">
         <v>4</v>
       </c>
       <c r="N44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>3.1956</v>
+        <v>3.1498</v>
       </c>
     </row>
     <row r="45">
@@ -3256,11 +3256,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>31/08/2024</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -3269,12 +3269,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3284,14 +3284,14 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I45" t="n">
         <v>4</v>
       </c>
       <c r="J45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K45" t="n">
         <v>3</v>
@@ -3300,18 +3300,18 @@
         <v>3</v>
       </c>
       <c r="M45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N45" t="n">
         <v>3</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P45" t="n">
-        <v>3.1498</v>
+        <v>3.1271</v>
       </c>
     </row>
     <row r="46">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>31/08/2024</t>
+          <t>05/05/2024</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3333,49 +3333,49 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I46" t="n">
         <v>4</v>
       </c>
       <c r="J46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K46" t="n">
         <v>3</v>
       </c>
       <c r="L46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M46" t="n">
         <v>3</v>
       </c>
       <c r="N46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.1271</v>
+        <v>3.1161</v>
       </c>
     </row>
     <row r="47">
@@ -3384,20 +3384,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>05/05/2024</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3412,11 +3412,11 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J47" t="n">
         <v>2</v>
@@ -3425,10 +3425,10 @@
         <v>3</v>
       </c>
       <c r="L47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N47" t="n">
         <v>5</v>
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>3.1161</v>
+        <v>3.092</v>
       </c>
     </row>
     <row r="48">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -3456,37 +3456,37 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J48" t="n">
         <v>2</v>
       </c>
       <c r="K48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
@@ -3495,15 +3495,15 @@
         <v>4</v>
       </c>
       <c r="N48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>3.092</v>
+        <v>3.0418</v>
       </c>
     </row>
     <row r="49">
@@ -3512,11 +3512,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3525,22 +3525,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I49" t="n">
@@ -3550,13 +3550,13 @@
         <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N49" t="n">
         <v>4</v>
@@ -3567,7 +3567,7 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>3.0418</v>
+        <v>3.0179</v>
       </c>
     </row>
     <row r="50">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -3584,54 +3584,54 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K50" t="n">
         <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>3.0179</v>
+        <v>2.9979</v>
       </c>
     </row>
     <row r="51">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>26/04/2025</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -3648,54 +3648,54 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K51" t="n">
         <v>3</v>
       </c>
       <c r="L51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>2.9979</v>
+        <v>2.9534</v>
       </c>
     </row>
     <row r="52">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3717,49 +3717,49 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I52" t="n">
         <v>4</v>
       </c>
       <c r="J52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2.9534</v>
+        <v>2.9471</v>
       </c>
     </row>
     <row r="53">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>20/09/2025</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -3806,24 +3806,24 @@
         <v>3</v>
       </c>
       <c r="K53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M53" t="n">
         <v>3</v>
       </c>
       <c r="N53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>E+E+D</t>
         </is>
       </c>
       <c r="P53" t="n">
-        <v>2.9471</v>
+        <v>2.9307</v>
       </c>
     </row>
     <row r="54">
@@ -3832,11 +3832,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>20/09/2025</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3845,22 +3845,22 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -3873,21 +3873,21 @@
         <v>3</v>
       </c>
       <c r="L54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>E+E+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2.9307</v>
+        <v>2.8708</v>
       </c>
     </row>
     <row r="55">
@@ -3896,11 +3896,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>17/09/2025</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -3909,7 +3909,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>17/09/2025</t>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3973,22 +3973,22 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -4001,7 +4001,7 @@
         <v>3</v>
       </c>
       <c r="L56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M56" t="n">
         <v>2</v>
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2.8708</v>
+        <v>2.8446</v>
       </c>
     </row>
     <row r="57">
@@ -4024,39 +4024,39 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J57" t="n">
         <v>3</v>
@@ -4065,21 +4065,21 @@
         <v>3</v>
       </c>
       <c r="L57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M57" t="n">
         <v>2</v>
       </c>
       <c r="N57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.8446</v>
+        <v>2.8419</v>
       </c>
     </row>
     <row r="58">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>15/02/2026</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -4096,54 +4096,54 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>Quartas</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N58" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>D+D+D</t>
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2.8419</v>
+        <v>2.8072</v>
       </c>
     </row>
     <row r="59">
@@ -4152,62 +4152,62 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>15/02/2026</t>
+          <t>16/07/2025</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Quartas</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>D+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2.8072</v>
+        <v>2.7507</v>
       </c>
     </row>
     <row r="60">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>16/07/2025</t>
+          <t>29/07/2025</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -4224,54 +4224,54 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J60" t="n">
         <v>3</v>
       </c>
       <c r="K60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L60" t="n">
         <v>4</v>
       </c>
       <c r="M60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N60" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2.7507</v>
+        <v>2.7437</v>
       </c>
     </row>
     <row r="61">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>29/07/2025</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -4293,17 +4293,17 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4321,21 +4321,21 @@
         <v>3</v>
       </c>
       <c r="L61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2.7437</v>
+        <v>2.5856</v>
       </c>
     </row>
     <row r="62">
@@ -4344,48 +4344,48 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>27/01/2024</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L62" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M62" t="n">
         <v>1</v>
@@ -4399,7 +4399,7 @@
         </is>
       </c>
       <c r="P62" t="n">
-        <v>2.5856</v>
+        <v>2.5587</v>
       </c>
     </row>
     <row r="63">
@@ -4408,11 +4408,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27/01/2024</t>
+          <t>11/01/2025</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -4421,12 +4421,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Maricá</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>11/01/2025</t>
+          <t>29/01/2025</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -4485,22 +4485,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Maricá</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I64" t="n">
@@ -4510,24 +4510,24 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L64" t="n">
         <v>3</v>
       </c>
       <c r="M64" t="n">
+        <v>4</v>
+      </c>
+      <c r="N64" t="n">
         <v>1</v>
       </c>
-      <c r="N64" t="n">
-        <v>4</v>
-      </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P64" t="n">
-        <v>2.5587</v>
+        <v>2.493</v>
       </c>
     </row>
     <row r="65">
@@ -4536,51 +4536,51 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>29/01/2025</t>
+          <t>21/04/2024</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J65" t="n">
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L65" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N65" t="n">
         <v>1</v>
@@ -4591,7 +4591,7 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>2.493</v>
+        <v>2.4408</v>
       </c>
     </row>
     <row r="66">
@@ -4600,11 +4600,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>21/04/2024</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -4613,22 +4613,22 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I66" t="n">
@@ -4641,7 +4641,7 @@
         <v>3</v>
       </c>
       <c r="L66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M66" t="n">
         <v>2</v>
@@ -4655,7 +4655,7 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>2.4408</v>
+        <v>2.4146</v>
       </c>
     </row>
     <row r="67">
@@ -4664,11 +4664,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>05/04/2025</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -4677,22 +4677,22 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Juventude</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -4705,7 +4705,7 @@
         <v>3</v>
       </c>
       <c r="L67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M67" t="n">
         <v>2</v>
@@ -4715,11 +4715,11 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P67" t="n">
-        <v>2.4146</v>
+        <v>2.3884</v>
       </c>
     </row>
     <row r="68">
@@ -4728,11 +4728,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>05/04/2025</t>
+          <t>18/04/2024</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Juventude</t>
+          <t>Atlético-GO</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -4751,12 +4751,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -4766,7 +4766,7 @@
         <v>2</v>
       </c>
       <c r="K68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L68" t="n">
         <v>3</v>
@@ -4779,11 +4779,11 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P68" t="n">
-        <v>2.3884</v>
+        <v>2.1822</v>
       </c>
     </row>
     <row r="69">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>18/04/2024</t>
+          <t>31/03/2024</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -4800,54 +4800,54 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Atlético-GO</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J69" t="n">
         <v>2</v>
       </c>
       <c r="K69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L69" t="n">
         <v>3</v>
       </c>
       <c r="M69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P69" t="n">
-        <v>2.1822</v>
+        <v>2.1463</v>
       </c>
     </row>
     <row r="70">
@@ -4856,11 +4856,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>31/03/2024</t>
+          <t>21/01/2026</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -4869,22 +4869,22 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I70" t="n">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>24/01/2026</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -4933,22 +4933,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I71" t="n">
@@ -4984,7 +4984,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>24/01/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -4997,12 +4997,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Boavista</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>SEMIS - TR</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -5048,11 +5048,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>17/03/2024</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -5061,22 +5061,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Boavista</t>
+          <t>Sampaio Corrêa</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>SEMIS - TR</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I73" t="n">
@@ -5095,15 +5095,15 @@
         <v>1</v>
       </c>
       <c r="N73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>2.1463</v>
+        <v>2.0481</v>
       </c>
     </row>
     <row r="74">
@@ -5112,11 +5112,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>17/03/2024</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -5125,22 +5125,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Sampaio Corrêa</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>FINAL - TR</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I74" t="n">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P74" t="n">
@@ -5176,11 +5176,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>30/01/2024</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -5189,22 +5189,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Portuguesa</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>FINAL - TR</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I75" t="n">
@@ -5214,24 +5214,24 @@
         <v>2</v>
       </c>
       <c r="K75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L75" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M75" t="n">
         <v>1</v>
       </c>
       <c r="N75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P75" t="n">
-        <v>2.0481</v>
+        <v>1.8877</v>
       </c>
     </row>
     <row r="76">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>30/01/2024</t>
+          <t>26/01/2025</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Portuguesa</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5263,12 +5263,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="I76" t="n">
@@ -5278,24 +5278,24 @@
         <v>2</v>
       </c>
       <c r="K76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M76" t="n">
         <v>1</v>
       </c>
       <c r="N76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P76" t="n">
-        <v>1.8877</v>
+        <v>1.8517</v>
       </c>
     </row>
     <row r="77">
@@ -5304,7 +5304,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>26/01/2025</t>
+          <t>14/01/2025</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -5317,22 +5317,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Portuguesa</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -5345,7 +5345,7 @@
         <v>3</v>
       </c>
       <c r="L77" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M77" t="n">
         <v>1</v>
@@ -5359,7 +5359,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>1.8517</v>
+        <v>1.7993</v>
       </c>
     </row>
     <row r="78">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>14/01/2025</t>
+          <t>22/01/2025</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -5381,22 +5381,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Portuguesa</t>
+          <t>Volta Redonda</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I78" t="n">
@@ -5406,10 +5406,10 @@
         <v>2</v>
       </c>
       <c r="K78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M78" t="n">
         <v>1</v>
@@ -5423,7 +5423,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>1.7993</v>
+        <v>1.6455</v>
       </c>
     </row>
     <row r="79">
@@ -5432,11 +5432,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>22/01/2025</t>
+          <t>17/01/2024</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -5445,12 +5445,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Volta Redonda</t>
+          <t>Madureira</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I79" t="n">
@@ -5470,7 +5470,7 @@
         <v>2</v>
       </c>
       <c r="K79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L79" t="n">
         <v>3</v>
@@ -5478,17 +5478,9 @@
       <c r="M79" t="n">
         <v>1</v>
       </c>
-      <c r="N79" t="n">
-        <v>1</v>
-      </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>V+D+D</t>
-        </is>
-      </c>
-      <c r="P79" t="n">
-        <v>1.6455</v>
-      </c>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -5496,7 +5488,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>17/01/2024</t>
+          <t>20/01/2024</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -5509,22 +5501,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Madureira</t>
+          <t>Bangu</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I80" t="n">
@@ -5534,7 +5526,7 @@
         <v>2</v>
       </c>
       <c r="K80" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L80" t="n">
         <v>3</v>
@@ -5545,62 +5537,6 @@
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>20/01/2024</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Carioca</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Bangu</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="I81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J81" t="n">
-        <v>2</v>
-      </c>
-      <c r="K81" t="n">
-        <v>5</v>
-      </c>
-      <c r="L81" t="n">
-        <v>3</v>
-      </c>
-      <c r="M81" t="n">
-        <v>1</v>
-      </c>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
AHP: ajustes de classificação e horários
- Libertadores: horário mínimo 4 (antes alguns eram 3)
- Red Bull Bragantino: grandeza 2 → 3
- Carioca: horário 20:30 limitado a 2
- Pearson r: 0.806 → 0.825 | Spearman r: 0.817 → 0.838

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>06/03/2024</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1152,54 +1152,54 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
         <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M12" t="n">
         <v>3</v>
       </c>
       <c r="N12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.8975</v>
+        <v>3.9154</v>
       </c>
     </row>
     <row r="13">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>08/05/2024</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1216,40 +1216,40 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
         <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M13" t="n">
         <v>3</v>
@@ -1263,7 +1263,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>3.8172</v>
+        <v>3.8975</v>
       </c>
     </row>
     <row r="14">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1285,12 +1285,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1316,18 +1316,18 @@
         <v>5</v>
       </c>
       <c r="M14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>3.8051</v>
+        <v>3.8172</v>
       </c>
     </row>
     <row r="15">
@@ -1336,25 +1336,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05/11/2025</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1364,34 +1364,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M15" t="n">
         <v>4</v>
       </c>
       <c r="N15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>3.6956</v>
+        <v>3.8051</v>
       </c>
     </row>
     <row r="16">
@@ -1400,11 +1400,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>03/04/2024</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1413,22 +1413,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Junior de Barranquilla</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1438,24 +1438,24 @@
         <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M16" t="n">
         <v>3</v>
       </c>
       <c r="N16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>3.6928</v>
+        <v>3.7092</v>
       </c>
     </row>
     <row r="17">
@@ -1464,11 +1464,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1477,49 +1477,49 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I17" t="n">
         <v>4</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>3.6901</v>
+        <v>3.6956</v>
       </c>
     </row>
     <row r="18">
@@ -1528,62 +1528,62 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>17/08/2025</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J18" t="n">
         <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>3.6584</v>
+        <v>3.6928</v>
       </c>
     </row>
     <row r="19">
@@ -1592,39 +1592,39 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06/03/2024</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J19" t="n">
         <v>3</v>
@@ -1636,18 +1636,18 @@
         <v>5</v>
       </c>
       <c r="M19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>3.6329</v>
+        <v>3.6901</v>
       </c>
     </row>
     <row r="20">
@@ -1656,11 +1656,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05/11/2024</t>
+          <t>17/08/2025</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1669,49 +1669,49 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I20" t="n">
         <v>4</v>
       </c>
       <c r="J20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M20" t="n">
         <v>4</v>
       </c>
       <c r="N20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>3.509</v>
+        <v>3.6584</v>
       </c>
     </row>
     <row r="21">
@@ -1720,62 +1720,62 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Universitario</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J21" t="n">
         <v>3</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" t="n">
         <v>4</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>3.5078</v>
+        <v>3.611</v>
       </c>
     </row>
     <row r="22">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>03/04/2024</t>
+          <t>14/08/2025</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1797,22 +1797,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Junior de Barranquilla</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1822,24 +1822,24 @@
         <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
       </c>
       <c r="N22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P22" t="n">
-        <v>3.503</v>
+        <v>3.5848</v>
       </c>
     </row>
     <row r="23">
@@ -1848,11 +1848,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>22/11/2025</t>
+          <t>05/11/2024</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1861,22 +1861,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Grêmio</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -1886,24 +1886,24 @@
         <v>4</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N23" t="n">
         <v>4</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>3.4851</v>
+        <v>3.509</v>
       </c>
     </row>
     <row r="24">
@@ -1912,62 +1912,62 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>30/07/2024</t>
+          <t>26/07/2025</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>3.4386</v>
+        <v>3.5078</v>
       </c>
     </row>
     <row r="25">
@@ -1976,62 +1976,62 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>22/11/2025</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aurora</t>
+          <t>Grêmio</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>3.4365</v>
+        <v>3.4851</v>
       </c>
     </row>
     <row r="26">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>17/07/2024</t>
+          <t>30/07/2024</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -2048,22 +2048,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2072,30 +2072,30 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J26" t="n">
         <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
         <v>4</v>
       </c>
       <c r="M26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P26" t="n">
-        <v>3.426</v>
+        <v>3.4386</v>
       </c>
     </row>
     <row r="27">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14/09/2024</t>
+          <t>28/02/2024</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -2112,54 +2112,54 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Aurora</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J27" t="n">
         <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N27" t="n">
         <v>3</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>3.4096</v>
+        <v>3.4365</v>
       </c>
     </row>
     <row r="28">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -2176,22 +2176,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Universitario</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2200,30 +2200,30 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J28" t="n">
         <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M28" t="n">
         <v>3</v>
       </c>
       <c r="N28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>3.4048</v>
+        <v>3.4288</v>
       </c>
     </row>
     <row r="29">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>23/11/2024</t>
+          <t>17/07/2024</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -2245,49 +2245,49 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I29" t="n">
         <v>4</v>
       </c>
       <c r="J29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>3.3869</v>
+        <v>3.426</v>
       </c>
     </row>
     <row r="30">
@@ -2296,39 +2296,39 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14/08/2025</t>
+          <t>14/09/2024</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J30" t="n">
         <v>3</v>
@@ -2337,21 +2337,21 @@
         <v>3</v>
       </c>
       <c r="L30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>3.3786</v>
+        <v>3.4096</v>
       </c>
     </row>
     <row r="31">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>19/06/2024</t>
+          <t>23/11/2024</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -2373,49 +2373,49 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Athlético</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I31" t="n">
         <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K31" t="n">
         <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M31" t="n">
         <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P31" t="n">
-        <v>3.3497</v>
+        <v>3.3869</v>
       </c>
     </row>
     <row r="32">
@@ -2424,11 +2424,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>19/06/2024</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2437,49 +2437,49 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Athlético</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I32" t="n">
         <v>4</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K32" t="n">
         <v>3</v>
       </c>
       <c r="L32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M32" t="n">
         <v>3</v>
       </c>
       <c r="N32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>3.3345</v>
+        <v>3.3497</v>
       </c>
     </row>
     <row r="33">
@@ -2488,11 +2488,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>20/07/2024</t>
+          <t>18/11/2025</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2501,49 +2501,49 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Sport</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I33" t="n">
         <v>4</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K33" t="n">
         <v>3</v>
       </c>
       <c r="L33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M33" t="n">
         <v>3</v>
       </c>
       <c r="N33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>3.3235</v>
+        <v>3.3345</v>
       </c>
     </row>
     <row r="34">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>18/02/2024</t>
+          <t>20/07/2024</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2560,54 +2560,54 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
         <v>3</v>
       </c>
       <c r="M34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3.308</v>
+        <v>3.3235</v>
       </c>
     </row>
     <row r="35">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>27/07/2024</t>
+          <t>18/02/2024</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2624,37 +2624,37 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K35" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L35" t="n">
         <v>3</v>
@@ -2663,15 +2663,15 @@
         <v>4</v>
       </c>
       <c r="N35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P35" t="n">
-        <v>3.3016</v>
+        <v>3.308</v>
       </c>
     </row>
     <row r="36">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07/07/2024</t>
+          <t>27/07/2024</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2693,22 +2693,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -2718,13 +2718,13 @@
         <v>3</v>
       </c>
       <c r="K36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N36" t="n">
         <v>4</v>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>3.2777</v>
+        <v>3.3016</v>
       </c>
     </row>
     <row r="37">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>16/04/2025</t>
+          <t>07/07/2024</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2757,49 +2757,49 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I37" t="n">
         <v>4</v>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K37" t="n">
         <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N37" t="n">
         <v>4</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>3.2742</v>
+        <v>3.2777</v>
       </c>
     </row>
     <row r="38">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>18/08/2024</t>
+          <t>16/04/2025</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2821,17 +2821,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2843,27 +2843,27 @@
         <v>4</v>
       </c>
       <c r="J38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
         <v>3</v>
       </c>
       <c r="L38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M38" t="n">
         <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>3.2656</v>
+        <v>3.2742</v>
       </c>
     </row>
     <row r="39">
@@ -2872,11 +2872,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04/06/2025</t>
+          <t>18/08/2024</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2885,22 +2885,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -2913,21 +2913,21 @@
         <v>3</v>
       </c>
       <c r="L39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>3.2515</v>
+        <v>3.2656</v>
       </c>
     </row>
     <row r="40">
@@ -2936,25 +2936,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>04/06/2025</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Nacional de Potosí</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2° FASE</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2964,34 +2964,34 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40" t="n">
         <v>3</v>
       </c>
       <c r="K40" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>3.2401</v>
+        <v>3.2515</v>
       </c>
     </row>
     <row r="41">
@@ -3000,25 +3000,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>15/10/2025</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Nacional de Potosí</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>2° FASE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3028,23 +3028,23 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J41" t="n">
         <v>3</v>
       </c>
       <c r="K41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N41" t="n">
         <v>1</v>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>3.2394</v>
+        <v>3.2401</v>
       </c>
     </row>
     <row r="42">
@@ -3064,39 +3064,39 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>15/10/2025</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J42" t="n">
         <v>3</v>
@@ -3108,18 +3108,18 @@
         <v>4</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N42" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3.2226</v>
+        <v>3.2394</v>
       </c>
     </row>
     <row r="43">
@@ -3128,25 +3128,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>29/07/2025</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3156,34 +3156,34 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>3.1956</v>
+        <v>3.2324</v>
       </c>
     </row>
     <row r="44">
@@ -3192,51 +3192,51 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Carabobo</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N44" t="n">
         <v>3</v>
@@ -3247,7 +3247,7 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>3.1498</v>
+        <v>3.2041</v>
       </c>
     </row>
     <row r="45">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>31/08/2024</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -3269,49 +3269,49 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I45" t="n">
         <v>4</v>
       </c>
       <c r="J45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K45" t="n">
         <v>3</v>
       </c>
       <c r="L45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P45" t="n">
-        <v>3.1271</v>
+        <v>3.1956</v>
       </c>
     </row>
     <row r="46">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>05/05/2024</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3333,49 +3333,49 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I46" t="n">
         <v>4</v>
       </c>
       <c r="J46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K46" t="n">
         <v>3</v>
       </c>
       <c r="L46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M46" t="n">
         <v>3</v>
       </c>
       <c r="N46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.1161</v>
+        <v>3.1533</v>
       </c>
     </row>
     <row r="47">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01/02/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -3392,22 +3392,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J47" t="n">
         <v>2</v>
@@ -3431,15 +3431,15 @@
         <v>4</v>
       </c>
       <c r="N47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P47" t="n">
-        <v>3.092</v>
+        <v>3.1498</v>
       </c>
     </row>
     <row r="48">
@@ -3448,11 +3448,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/01/2026</t>
+          <t>31/08/2024</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -3461,49 +3461,49 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I48" t="n">
         <v>4</v>
       </c>
       <c r="J48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L48" t="n">
         <v>3</v>
       </c>
       <c r="M48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P48" t="n">
-        <v>3.0418</v>
+        <v>3.1271</v>
       </c>
     </row>
     <row r="49">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>11/05/2025</t>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -3525,49 +3525,49 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I49" t="n">
         <v>4</v>
       </c>
       <c r="J49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
         <v>3</v>
       </c>
       <c r="L49" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M49" t="n">
         <v>3</v>
       </c>
       <c r="N49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P49" t="n">
-        <v>3.0179</v>
+        <v>3.1271</v>
       </c>
     </row>
     <row r="50">
@@ -3576,62 +3576,62 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>05/05/2024</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Carabobo</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K50" t="n">
         <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2.9979</v>
+        <v>3.1161</v>
       </c>
     </row>
     <row r="51">
@@ -3640,62 +3640,62 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>26/04/2025</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Sulamericana</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Caracas</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M51" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P51" t="n">
-        <v>2.9534</v>
+        <v>3.0481</v>
       </c>
     </row>
     <row r="52">
@@ -3704,11 +3704,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>29/01/2026</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -3717,17 +3717,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3739,27 +3739,27 @@
         <v>4</v>
       </c>
       <c r="J52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="n">
         <v>2</v>
       </c>
       <c r="L52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2.9471</v>
+        <v>3.0418</v>
       </c>
     </row>
     <row r="53">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>20/09/2025</t>
+          <t>11/05/2025</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3781,49 +3781,49 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Atlético-MG</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="I53" t="n">
         <v>4</v>
       </c>
       <c r="J53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K53" t="n">
         <v>3</v>
       </c>
       <c r="L53" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M53" t="n">
         <v>3</v>
       </c>
       <c r="N53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>E+E+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P53" t="n">
-        <v>2.9307</v>
+        <v>3.0179</v>
       </c>
     </row>
     <row r="54">
@@ -3832,11 +3832,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>26/04/2025</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -3845,49 +3845,49 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="I54" t="n">
         <v>4</v>
       </c>
       <c r="J54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K54" t="n">
         <v>3</v>
       </c>
       <c r="L54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N54" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2.8708</v>
+        <v>2.9534</v>
       </c>
     </row>
     <row r="55">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>17/09/2025</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3909,12 +3909,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -3934,13 +3934,13 @@
         <v>3</v>
       </c>
       <c r="K55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L55" t="n">
         <v>4</v>
       </c>
       <c r="M55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N55" t="n">
         <v>3</v>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>2.8708</v>
+        <v>2.9471</v>
       </c>
     </row>
     <row r="56">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>30/08/2025</t>
+          <t>20/09/2025</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Atlético-MG</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4004,18 +4004,18 @@
         <v>3</v>
       </c>
       <c r="M56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N56" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>E+E+D</t>
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2.8446</v>
+        <v>2.9307</v>
       </c>
     </row>
     <row r="57">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>01/02/2026</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4032,54 +4032,54 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Sulamericana</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Caracas</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N57" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2.8419</v>
+        <v>2.8858</v>
       </c>
     </row>
     <row r="58">
@@ -4088,62 +4088,62 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>15/02/2026</t>
+          <t>17/09/2025</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Carioca</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Quartas</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M58" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N58" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>D+D+D</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2.8072</v>
+        <v>2.8708</v>
       </c>
     </row>
     <row r="59">
@@ -4152,62 +4152,62 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>16/07/2025</t>
+          <t>15/02/2026</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Carioca</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Vitória</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>Quartas</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>D+D+D</t>
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2.7507</v>
+        <v>2.8072</v>
       </c>
     </row>
     <row r="60">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>29/07/2025</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -4229,17 +4229,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4254,24 +4254,24 @@
         <v>3</v>
       </c>
       <c r="K60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L60" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N60" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2.7437</v>
+        <v>2.7918</v>
       </c>
     </row>
     <row r="61">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>16/07/2025</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -4288,17 +4288,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Vitória</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4308,34 +4308,34 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J61" t="n">
         <v>3</v>
       </c>
       <c r="K61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M61" t="n">
+        <v>3</v>
+      </c>
+      <c r="N61" t="n">
         <v>1</v>
       </c>
-      <c r="N61" t="n">
-        <v>4</v>
-      </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2.5856</v>
+        <v>2.7507</v>
       </c>
     </row>
     <row r="62">

</xml_diff>

<commit_message>
AHP: Libertadores OITAVAS = 4 (override de fase por campeonato)
Pearson r: 0.825 → 0.832 | Spearman r: 0.838 → 0.844

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -952,11 +952,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -965,17 +965,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -987,27 +987,27 @@
         <v>5</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
         <v>5</v>
       </c>
       <c r="L9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
         <v>4</v>
       </c>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>3.9753</v>
+        <v>4.0649</v>
       </c>
     </row>
     <row r="10">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>03/08/2025</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1024,31 +1024,31 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" t="n">
         <v>3</v>
@@ -1057,21 +1057,21 @@
         <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M10" t="n">
         <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>3.9726</v>
+        <v>3.9753</v>
       </c>
     </row>
     <row r="11">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>03/08/2025</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1093,12 +1093,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1115,7 +1115,7 @@
         <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>5</v>
@@ -1127,15 +1127,15 @@
         <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>3.9378</v>
+        <v>3.9726</v>
       </c>
     </row>
     <row r="12">
@@ -1144,42 +1144,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06/03/2024</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K12" t="n">
         <v>5</v>
@@ -1188,18 +1188,18 @@
         <v>5</v>
       </c>
       <c r="M12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.9154</v>
+        <v>3.9378</v>
       </c>
     </row>
     <row r="13">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>06/03/2024</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1216,54 +1216,54 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
         <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M13" t="n">
         <v>3</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>3.8975</v>
+        <v>3.9154</v>
       </c>
     </row>
     <row r="14">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>08/05/2024</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1280,40 +1280,40 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K14" t="n">
         <v>5</v>
       </c>
       <c r="L14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
         <v>3</v>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>3.8172</v>
+        <v>3.8975</v>
       </c>
     </row>
     <row r="15">
@@ -1336,11 +1336,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>14/08/2025</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1359,39 +1359,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I15" t="n">
         <v>5</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>3.8051</v>
+        <v>3.8446</v>
       </c>
     </row>
     <row r="16">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>03/04/2024</t>
+          <t>08/05/2024</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Junior de Barranquilla</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1438,7 +1438,7 @@
         <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
         <v>5</v>
@@ -1447,15 +1447,15 @@
         <v>3</v>
       </c>
       <c r="N16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>3.7092</v>
+        <v>3.8172</v>
       </c>
     </row>
     <row r="17">
@@ -1464,25 +1464,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05/11/2025</t>
+          <t>03/04/2024</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>Junior de Barranquilla</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1492,34 +1492,34 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>3.6956</v>
+        <v>3.7092</v>
       </c>
     </row>
     <row r="18">
@@ -1528,51 +1528,51 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Barcelona de Guayaquil</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3° Fase</t>
+          <t>32</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
         <v>4</v>
       </c>
       <c r="M18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" t="n">
         <v>3</v>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>3.6928</v>
+        <v>3.6956</v>
       </c>
     </row>
     <row r="19">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1600,31 +1600,31 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Barcelona de Guayaquil</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3° Fase</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J19" t="n">
         <v>3</v>
@@ -1633,21 +1633,21 @@
         <v>5</v>
       </c>
       <c r="L19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M19" t="n">
         <v>3</v>
       </c>
       <c r="N19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>3.6901</v>
+        <v>3.6928</v>
       </c>
     </row>
     <row r="20">
@@ -1656,11 +1656,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>17/08/2025</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1669,12 +1669,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1694,24 +1694,24 @@
         <v>3</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L20" t="n">
         <v>5</v>
       </c>
       <c r="M20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>3.6584</v>
+        <v>3.6901</v>
       </c>
     </row>
     <row r="21">
@@ -1720,62 +1720,62 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>17/08/2025</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Universitario</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J21" t="n">
         <v>3</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
         <v>5</v>
       </c>
       <c r="M21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>3.611</v>
+        <v>3.6584</v>
       </c>
     </row>
     <row r="22">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>14/08/2025</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1797,17 +1797,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Universitario</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1825,7 +1825,7 @@
         <v>4</v>
       </c>
       <c r="L22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>3.5848</v>
+        <v>3.611</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
AHP: Libertadores OITAVAS/QUARTAS/SEMIS = 5
Pearson r: 0.832 → 0.835 | Spearman r: 0.844 → 0.846

https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/AHP_Pontuacao_Partidas.xlsx
+++ b/AHP_Pontuacao_Partidas.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>08/12/2024</t>
+          <t>18/09/2024</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -512,7 +512,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -522,21 +522,21 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>QUARTAS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J2" t="n">
         <v>5</v>
@@ -551,15 +551,15 @@
         <v>4</v>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>4.5904</v>
+        <v>4.6193</v>
       </c>
     </row>
     <row r="3">
@@ -568,7 +568,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>23/10/2024</t>
+          <t>08/12/2024</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -576,31 +576,31 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Peñarol</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SEMIS</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3" t="n">
         <v>5</v>
@@ -615,15 +615,15 @@
         <v>4</v>
       </c>
       <c r="N3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>4.5211</v>
+        <v>4.5904</v>
       </c>
     </row>
     <row r="4">
@@ -632,7 +632,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>18/09/2024</t>
+          <t>23/10/2024</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -645,12 +645,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Peñarol</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>SEMIS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -667,7 +667,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4" t="n">
         <v>5</v>
@@ -679,15 +679,15 @@
         <v>4</v>
       </c>
       <c r="N4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>4.3595</v>
+        <v>4.5211</v>
       </c>
     </row>
     <row r="5">
@@ -696,30 +696,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>27/02/2025</t>
+          <t>14/08/2024</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Recopa</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Racing</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>FINAL</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -737,7 +737,7 @@
         <v>5</v>
       </c>
       <c r="L5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M5" t="n">
         <v>4</v>
@@ -747,11 +747,11 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>E+D+D</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4.2985</v>
+        <v>4.3247</v>
       </c>
     </row>
     <row r="6">
@@ -760,7 +760,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07/12/2025</t>
+          <t>27/02/2025</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -768,31 +768,31 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Recopa</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Racing</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>FINAL</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
         <v>5</v>
@@ -801,21 +801,21 @@
         <v>5</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>V+E+E</t>
+          <t>E+D+D</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>4.1115</v>
+        <v>4.2985</v>
       </c>
     </row>
     <row r="7">
@@ -824,7 +824,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>14/05/2025</t>
+          <t>07/12/2025</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -832,34 +832,34 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Estudiantes</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
         <v>5</v>
@@ -868,18 +868,18 @@
         <v>5</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+E+E</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>4.0997</v>
+        <v>4.1115</v>
       </c>
     </row>
     <row r="8">
@@ -888,7 +888,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11/09/2025</t>
+          <t>14/08/2025</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -896,17 +896,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Copa do Brasil</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Vasco da Gama</t>
+          <t>LDU Quito</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>QUARTAS</t>
+          <t>OITAVAS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -916,34 +916,34 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
         <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8" t="n">
         <v>4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>4.0791</v>
+        <v>4.1044</v>
       </c>
     </row>
     <row r="9">
@@ -952,11 +952,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14/08/2024</t>
+          <t>14/05/2025</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -965,12 +965,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Estudiantes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -987,7 +987,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
         <v>5</v>
@@ -999,15 +999,15 @@
         <v>4</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+D</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>4.0649</v>
+        <v>4.0997</v>
       </c>
     </row>
     <row r="10">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>11/09/2025</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1024,22 +1024,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Copa do Brasil</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Universidad de Chile</t>
+          <t>Vasco da Gama</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>QUARTAS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Terça-feira</t>
+          <t>Quinta-feira</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1048,10 +1048,10 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
         <v>5</v>
@@ -1063,15 +1063,15 @@
         <v>4</v>
       </c>
       <c r="N10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>V+E+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>3.9753</v>
+        <v>4.0791</v>
       </c>
     </row>
     <row r="11">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>03/08/2025</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1088,31 +1088,31 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Universidad de Chile</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Domingo</t>
+          <t>Terça-feira</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>
@@ -1121,21 +1121,21 @@
         <v>5</v>
       </c>
       <c r="L11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M11" t="n">
         <v>4</v>
       </c>
       <c r="N11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>V+V+E</t>
+          <t>V+E+D</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>3.9726</v>
+        <v>3.9753</v>
       </c>
     </row>
     <row r="12">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>26/10/2025</t>
+          <t>03/08/2025</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1179,7 +1179,7 @@
         <v>4</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
         <v>5</v>
@@ -1191,15 +1191,15 @@
         <v>4</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>V+D+D</t>
+          <t>V+V+E</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>3.9378</v>
+        <v>3.9726</v>
       </c>
     </row>
     <row r="13">
@@ -1208,42 +1208,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06/03/2024</t>
+          <t>26/10/2025</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3° FASE</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Quarta-feira</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
         <v>5</v>
@@ -1252,18 +1252,18 @@
         <v>5</v>
       </c>
       <c r="M13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>V+V+V</t>
+          <t>V+D+D</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>3.9154</v>
+        <v>3.9378</v>
       </c>
     </row>
     <row r="14">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09/11/2024</t>
+          <t>06/03/2024</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1280,54 +1280,54 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Brasileirão</t>
+          <t>Libertadores</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Cuiabá</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>3° FASE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Quarta-feira</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
         <v>5</v>
       </c>
       <c r="L14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M14" t="n">
         <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>V+V+D</t>
+          <t>V+V+V</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>3.8975</v>
+        <v>3.9154</v>
       </c>
     </row>
     <row r="15">
@@ -1336,48 +1336,48 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14/08/2025</t>
+          <t>09/11/2024</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Libertadores</t>
+          <t>Brasileirão</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LDU Quito</t>
+          <t>Cuiabá</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>OITAVAS</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Quinta-feira</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J15" t="n">
         <v>4</v>
       </c>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
         <v>3</v>
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>3.8446</v>
+        <v>3.8975</v>
       </c>
     </row>
     <row r="16">

</xml_diff>